<commit_message>
Expand six-city dish data, docs, and store photo tooling.
Sync spreadsheets, AMap enrichment artifacts, UI tweaks, doc-link audit script, and KL/Melaka photo renames.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/src/data/restaurants.xlsx
+++ b/src/data/restaurants.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD222"/>
+  <dimension ref="A1:AE222"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -494,6 +494,9 @@
       <c r="AD1" t="str">
         <v>record_scope</v>
       </c>
+      <c r="AE1" t="str">
+        <v>cuisine</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -517,6 +520,12 @@
       <c r="G2" t="str">
         <v>仙生生寿司专门店(中山店)</v>
       </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
       <c r="J2" t="str">
         <v>日料</v>
       </c>
@@ -603,6 +612,12 @@
       <c r="G3" t="str">
         <v>皇家面点(顺阳街)</v>
       </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
       <c r="J3" t="str">
         <v>糕点</v>
       </c>
@@ -689,6 +704,12 @@
       <c r="G4" t="str">
         <v>日月昇海鲜码头(民主广场店)</v>
       </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
       <c r="J4" t="str">
         <v>海鲜</v>
       </c>
@@ -775,6 +796,12 @@
       <c r="G5" t="str">
         <v>WUYOO冰奶大连中山店</v>
       </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
       <c r="J5" t="str">
         <v>奶茶</v>
       </c>
@@ -861,6 +888,12 @@
       <c r="G6" t="str">
         <v>阿水的生鱼饭旗舰店(长江路店)</v>
       </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
       <c r="J6" t="str">
         <v>日料</v>
       </c>
@@ -947,6 +980,12 @@
       <c r="G7" t="str">
         <v>鹅记好吃店</v>
       </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
       <c r="J7" t="str">
         <v>甜品</v>
       </c>
@@ -1033,6 +1072,12 @@
       <c r="G8" t="str">
         <v>奉天玖福记沈阳鸡架(奥林匹克店)</v>
       </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
       <c r="J8" t="str">
         <v>东北菜</v>
       </c>
@@ -1119,6 +1164,12 @@
       <c r="G9" t="str">
         <v>東北灵丹·SUP(南山路超级萃取店)</v>
       </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
       <c r="J9" t="str">
         <v>咖啡</v>
       </c>
@@ -1205,6 +1256,12 @@
       <c r="G10" t="str">
         <v>王慧洁开口虾水饺·地道东北菜(银泰城店)</v>
       </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
       <c r="J10" t="str">
         <v>东北菜</v>
       </c>
@@ -1291,6 +1348,12 @@
       <c r="G11" t="str">
         <v>DIVECOFFEE2.0 南山店</v>
       </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
       <c r="J11" t="str">
         <v>咖啡</v>
       </c>
@@ -1377,6 +1440,12 @@
       <c r="G12" t="str">
         <v>岐迹正宗无水南瓜糕</v>
       </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
       <c r="J12" t="str">
         <v>糕点</v>
       </c>
@@ -1466,8 +1535,11 @@
       <c r="H13" t="str">
         <v>Dongmun Traditional Market</v>
       </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
       <c r="J13" t="str">
-        <v>小吃</v>
+        <v>街头小吃</v>
       </c>
       <c r="K13" t="str">
         <v>street-food</v>
@@ -1481,6 +1553,9 @@
       <c r="N13" t="str">
         <v>33.5115133</v>
       </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
       <c r="P13" t="str">
         <v>4.1</v>
       </c>
@@ -1525,6 +1600,9 @@
       </c>
       <c r="AD13" t="str">
         <v>branch</v>
+      </c>
+      <c r="AE13" t="str">
+        <v>街头小吃</v>
       </c>
     </row>
     <row r="14">
@@ -1549,6 +1627,9 @@
       <c r="G14" t="str">
         <v>牛岛花生冰淇淋</v>
       </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
       <c r="I14" t="str">
         <v>하고야까페</v>
       </c>
@@ -1567,11 +1648,20 @@
       <c r="N14" t="str">
         <v>33.513902</v>
       </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
       <c r="P14" t="str">
         <v>5</v>
       </c>
       <c r="Q14" t="str">
         <v>KRW</v>
+      </c>
+      <c r="R14" t="str">
+        <v/>
+      </c>
+      <c r="S14" t="str">
+        <v/>
       </c>
       <c r="T14" t="str">
         <v>google</v>
@@ -1632,6 +1722,9 @@
       <c r="H15" t="str">
         <v>Baek So Jeong</v>
       </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
       <c r="J15" t="str">
         <v>韩餐</v>
       </c>
@@ -1721,6 +1814,9 @@
       <c r="H16" t="str">
         <v>Haenyeo Gimbap Main Branch</v>
       </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
       <c r="J16" t="str">
         <v>韩餐</v>
       </c>
@@ -1807,6 +1903,9 @@
       <c r="G17" t="str">
         <v>咸德细花排骨</v>
       </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
       <c r="I17" t="str">
         <v>세화갈비함덕직영점</v>
       </c>
@@ -1988,6 +2087,9 @@
       <c r="G19" t="str">
         <v>24h土豆脊骨汤</v>
       </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
       <c r="I19" t="str">
         <v>24시뼈다귀감자탕</v>
       </c>
@@ -2077,6 +2179,9 @@
       <c r="G20" t="str">
         <v>梨花鸡爪1979</v>
       </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
       <c r="I20" t="str">
         <v>이화닭발1979</v>
       </c>
@@ -2103,6 +2208,9 @@
       </c>
       <c r="Q20" t="str">
         <v>CNY</v>
+      </c>
+      <c r="R20" t="str">
+        <v/>
       </c>
       <c r="S20" t="str">
         <v>+82 64-749-1979</v>
@@ -2160,6 +2268,9 @@
       <c r="F21" t="str">
         <v>compose-coffee</v>
       </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
       <c r="H21" t="str">
         <v>Compose Coffee</v>
       </c>
@@ -2192,6 +2303,9 @@
       </c>
       <c r="R21" t="str">
         <v>周一至周日 10:00–21:00</v>
+      </c>
+      <c r="S21" t="str">
+        <v/>
       </c>
       <c r="T21" t="str">
         <v>google</v>
@@ -2249,6 +2363,9 @@
       <c r="G22" t="str">
         <v>BHC炸鸡(莲洞店)</v>
       </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
       <c r="I22" t="str">
         <v>BHC치킨 연동점</v>
       </c>
@@ -2335,8 +2452,14 @@
       <c r="F23" t="str">
         <v>mega-coffee</v>
       </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
       <c r="H23" t="str">
         <v>Mega MGC Coffee Jeju Docheong Branch</v>
+      </c>
+      <c r="I23" t="str">
+        <v/>
       </c>
       <c r="J23" t="str">
         <v>咖啡</v>
@@ -2424,6 +2547,12 @@
       <c r="G24" t="str">
         <v>Baro猪蹄</v>
       </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
       <c r="J24" t="str">
         <v>韩餐</v>
       </c>
@@ -2510,6 +2639,9 @@
       <c r="G25" t="str">
         <v>济州黑猪</v>
       </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
       <c r="I25" t="str">
         <v>제주깜돈</v>
       </c>
@@ -2527,6 +2659,9 @@
       </c>
       <c r="N25" t="str">
         <v>33.5419042</v>
+      </c>
+      <c r="O25" t="str">
+        <v/>
       </c>
       <c r="P25" t="str">
         <v>4</v>
@@ -2606,7 +2741,7 @@
         <v>咖啡</v>
       </c>
       <c r="K26" t="str">
-        <v>co</v>
+        <v>coffee</v>
       </c>
       <c r="L26" t="str">
         <v>32 Jungmungwangwang-ro 110beon-gil, 특별자치도 Seogwipo, Jeju-do, 韩国</v>
@@ -2688,6 +2823,12 @@
       <c r="G27" t="str">
         <v>牛岛白沙滩猪排店</v>
       </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
       <c r="J27" t="str">
         <v>韩餐</v>
       </c>
@@ -2696,6 +2837,33 @@
       </c>
       <c r="L27" t="str">
         <v>连锁店</v>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
+      <c r="O27" t="str">
+        <v/>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
+      <c r="R27" t="str">
+        <v/>
+      </c>
+      <c r="S27" t="str">
+        <v/>
+      </c>
+      <c r="T27" t="str">
+        <v/>
+      </c>
+      <c r="U27" t="str">
+        <v/>
       </c>
       <c r="V27" t="str">
         <v>dine_in</v>
@@ -2747,6 +2915,12 @@
       <c r="G28" t="str">
         <v>CU便利店</v>
       </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
       <c r="J28" t="str">
         <v>零食</v>
       </c>
@@ -2755,6 +2929,33 @@
       </c>
       <c r="L28" t="str">
         <v>连锁店</v>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
+      <c r="N28" t="str">
+        <v/>
+      </c>
+      <c r="O28" t="str">
+        <v/>
+      </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+      <c r="Q28" t="str">
+        <v/>
+      </c>
+      <c r="R28" t="str">
+        <v/>
+      </c>
+      <c r="S28" t="str">
+        <v/>
+      </c>
+      <c r="T28" t="str">
+        <v/>
+      </c>
+      <c r="U28" t="str">
+        <v/>
       </c>
       <c r="V28" t="str">
         <v>takeout</v>
@@ -2806,6 +3007,12 @@
       <c r="G29" t="str">
         <v>GS25便利店</v>
       </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29" t="str">
+        <v/>
+      </c>
       <c r="J29" t="str">
         <v>零食</v>
       </c>
@@ -2814,6 +3021,33 @@
       </c>
       <c r="L29" t="str">
         <v>连锁店</v>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
+      <c r="N29" t="str">
+        <v/>
+      </c>
+      <c r="O29" t="str">
+        <v/>
+      </c>
+      <c r="P29" t="str">
+        <v/>
+      </c>
+      <c r="Q29" t="str">
+        <v/>
+      </c>
+      <c r="R29" t="str">
+        <v/>
+      </c>
+      <c r="S29" t="str">
+        <v/>
+      </c>
+      <c r="T29" t="str">
+        <v/>
+      </c>
+      <c r="U29" t="str">
+        <v/>
       </c>
       <c r="V29" t="str">
         <v>takeout</v>
@@ -2862,8 +3096,14 @@
       <c r="F30" t="str">
         <v>tr</v>
       </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
       <c r="H30" t="str">
         <v>The Tokyo Restaurant</v>
+      </c>
+      <c r="I30" t="str">
+        <v/>
       </c>
       <c r="J30" t="str">
         <v>甜品</v>
@@ -2948,8 +3188,14 @@
       <c r="F31" t="str">
         <v>vcr</v>
       </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
       <c r="H31" t="str">
         <v>VCR</v>
+      </c>
+      <c r="I31" t="str">
+        <v/>
       </c>
       <c r="J31" t="str">
         <v>咖啡</v>
@@ -3040,6 +3286,9 @@
       <c r="H32" t="str">
         <v>Hai Kah Lang</v>
       </c>
+      <c r="I32" t="str">
+        <v/>
+      </c>
       <c r="J32" t="str">
         <v>海鲜</v>
       </c>
@@ -3129,6 +3378,9 @@
       <c r="H33" t="str">
         <v>Oriental Kopi • Suria KLCC</v>
       </c>
+      <c r="I33" t="str">
+        <v/>
+      </c>
       <c r="J33" t="str">
         <v>东南亚菜</v>
       </c>
@@ -3212,9 +3464,15 @@
       <c r="F34" t="str">
         <v>boost</v>
       </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
       <c r="H34" t="str">
         <v>Boost Juice</v>
       </c>
+      <c r="I34" t="str">
+        <v/>
+      </c>
       <c r="J34" t="str">
         <v>奶茶</v>
       </c>
@@ -3224,6 +3482,12 @@
       <c r="L34" t="str">
         <v>连锁店</v>
       </c>
+      <c r="M34" t="str">
+        <v/>
+      </c>
+      <c r="N34" t="str">
+        <v/>
+      </c>
       <c r="O34">
         <v>25</v>
       </c>
@@ -3241,6 +3505,9 @@
       </c>
       <c r="T34" t="str">
         <v>google</v>
+      </c>
+      <c r="U34" t="str">
+        <v/>
       </c>
       <c r="V34" t="str">
         <v>takeout</v>
@@ -3289,9 +3556,15 @@
       <c r="F35" t="str">
         <v>lavender</v>
       </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
       <c r="H35" t="str">
         <v>Lavender Bakery</v>
       </c>
+      <c r="I35" t="str">
+        <v/>
+      </c>
       <c r="J35" t="str">
         <v>面包</v>
       </c>
@@ -3301,9 +3574,21 @@
       <c r="L35" t="str">
         <v>连锁店</v>
       </c>
+      <c r="M35" t="str">
+        <v/>
+      </c>
+      <c r="N35" t="str">
+        <v/>
+      </c>
+      <c r="O35" t="str">
+        <v/>
+      </c>
       <c r="P35">
         <v>3.9</v>
       </c>
+      <c r="Q35" t="str">
+        <v/>
+      </c>
       <c r="R35" t="str">
         <v>周一至周日 10:00–22:00</v>
       </c>
@@ -3312,6 +3597,9 @@
       </c>
       <c r="T35" t="str">
         <v>google</v>
+      </c>
+      <c r="U35" t="str">
+        <v/>
       </c>
       <c r="V35" t="str">
         <v>takeout</v>
@@ -3366,6 +3654,9 @@
       <c r="H36" t="str">
         <v>7-Eleven</v>
       </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
       <c r="J36" t="str">
         <v>零食</v>
       </c>
@@ -3375,6 +3666,12 @@
       <c r="L36" t="str">
         <v>连锁店</v>
       </c>
+      <c r="M36" t="str">
+        <v/>
+      </c>
+      <c r="N36" t="str">
+        <v/>
+      </c>
       <c r="O36">
         <v>31</v>
       </c>
@@ -3392,6 +3689,9 @@
       </c>
       <c r="T36" t="str">
         <v>google</v>
+      </c>
+      <c r="U36" t="str">
+        <v/>
       </c>
       <c r="V36" t="str">
         <v>takeout</v>
@@ -3440,8 +3740,14 @@
       <c r="F37" t="str">
         <v>abg22</v>
       </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
       <c r="H37" t="str">
         <v>Aaagain by Grounded 22</v>
+      </c>
+      <c r="I37" t="str">
+        <v/>
       </c>
       <c r="J37" t="str">
         <v>咖啡</v>
@@ -3532,6 +3838,9 @@
       <c r="H38" t="str">
         <v>DeXingLung Kopitiam</v>
       </c>
+      <c r="I38" t="str">
+        <v/>
+      </c>
       <c r="J38" t="str">
         <v>东南亚菜</v>
       </c>
@@ -3616,7 +3925,13 @@
         <v>sbt</v>
       </c>
       <c r="G39" t="str">
-        <v>十八梯板凳面(总店)</v>
+        <v>十八梯邓凳面(总店)</v>
+      </c>
+      <c r="H39" t="str">
+        <v/>
+      </c>
+      <c r="I39" t="str">
+        <v/>
       </c>
       <c r="J39" t="str">
         <v>面条</v>
@@ -3704,6 +4019,12 @@
       <c r="G40" t="str">
         <v>福兴老火锅(直营二分店)</v>
       </c>
+      <c r="H40" t="str">
+        <v/>
+      </c>
+      <c r="I40" t="str">
+        <v/>
+      </c>
       <c r="J40" t="str">
         <v>火锅</v>
       </c>
@@ -3790,6 +4111,12 @@
       <c r="G41" t="str">
         <v>民间粮仓·重庆菜(观音桥店重庆总店)</v>
       </c>
+      <c r="H41" t="str">
+        <v/>
+      </c>
+      <c r="I41" t="str">
+        <v/>
+      </c>
       <c r="J41" t="str">
         <v>川菜</v>
       </c>
@@ -3876,6 +4203,12 @@
       <c r="G42" t="str">
         <v>久鑫美蛙鱼头(弹子石店)</v>
       </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
+      <c r="I42" t="str">
+        <v/>
+      </c>
       <c r="J42" t="str">
         <v>火锅</v>
       </c>
@@ -3962,6 +4295,12 @@
       <c r="G43" t="str">
         <v>马房湾66号·江湖菜</v>
       </c>
+      <c r="H43" t="str">
+        <v/>
+      </c>
+      <c r="I43" t="str">
+        <v/>
+      </c>
       <c r="J43" t="str">
         <v>川菜</v>
       </c>
@@ -4048,6 +4387,12 @@
       <c r="G44" t="str">
         <v>四间火锅(上清寺老重庆店)</v>
       </c>
+      <c r="H44" t="str">
+        <v/>
+      </c>
+      <c r="I44" t="str">
+        <v/>
+      </c>
       <c r="J44" t="str">
         <v>火锅</v>
       </c>
@@ -4134,6 +4479,12 @@
       <c r="G45" t="str">
         <v>显芳面条(解放碑步行街店)</v>
       </c>
+      <c r="H45" t="str">
+        <v/>
+      </c>
+      <c r="I45" t="str">
+        <v/>
+      </c>
       <c r="J45" t="str">
         <v>面条</v>
       </c>
@@ -4220,6 +4571,12 @@
       <c r="G46" t="str">
         <v>超级李板凳面</v>
       </c>
+      <c r="H46" t="str">
+        <v/>
+      </c>
+      <c r="I46" t="str">
+        <v/>
+      </c>
       <c r="J46" t="str">
         <v>面条</v>
       </c>
@@ -4306,6 +4663,12 @@
       <c r="G47" t="str">
         <v>七妹糊辣辣(渝海大厦店)</v>
       </c>
+      <c r="H47" t="str">
+        <v/>
+      </c>
+      <c r="I47" t="str">
+        <v/>
+      </c>
       <c r="J47" t="str">
         <v>面条</v>
       </c>
@@ -4334,7 +4697,7 @@
         <v>周一至周日 07:00-20:00</v>
       </c>
       <c r="S47" t="str">
-        <v>13696464527;18375737176</v>
+        <v>13696464527；18375737176</v>
       </c>
       <c r="T47" t="str">
         <v>amap</v>
@@ -4392,6 +4755,12 @@
       <c r="G48" t="str">
         <v>姚脑壳乐山鲜烧牛肉</v>
       </c>
+      <c r="H48" t="str">
+        <v/>
+      </c>
+      <c r="I48" t="str">
+        <v/>
+      </c>
       <c r="J48" t="str">
         <v>火锅</v>
       </c>
@@ -4478,6 +4847,12 @@
       <c r="G49" t="str">
         <v>重庆吃山文化青年旅店</v>
       </c>
+      <c r="H49" t="str">
+        <v/>
+      </c>
+      <c r="I49" t="str">
+        <v/>
+      </c>
       <c r="J49" t="str">
         <v>其他</v>
       </c>
@@ -4493,6 +4868,9 @@
       <c r="N49">
         <v>29.561122</v>
       </c>
+      <c r="O49" t="str">
+        <v/>
+      </c>
       <c r="P49">
         <v>4.9</v>
       </c>
@@ -4503,7 +4881,7 @@
         <v>全天开放</v>
       </c>
       <c r="S49" t="str">
-        <v>023-63005556;19922839130</v>
+        <v>023-63005556；19922839130</v>
       </c>
       <c r="T49" t="str">
         <v>amap</v>
@@ -4561,6 +4939,12 @@
       <c r="G50" t="str">
         <v>啥子巷巷大汤圆</v>
       </c>
+      <c r="H50" t="str">
+        <v/>
+      </c>
+      <c r="I50" t="str">
+        <v/>
+      </c>
       <c r="J50" t="str">
         <v>甜品</v>
       </c>
@@ -4647,6 +5031,12 @@
       <c r="G51" t="str">
         <v>起风咖啡</v>
       </c>
+      <c r="H51" t="str">
+        <v/>
+      </c>
+      <c r="I51" t="str">
+        <v/>
+      </c>
       <c r="J51" t="str">
         <v>咖啡</v>
       </c>
@@ -4733,6 +5123,12 @@
       <c r="G52" t="str">
         <v>老重庆豆花饭(星天广场店)</v>
       </c>
+      <c r="H52" t="str">
+        <v/>
+      </c>
+      <c r="I52" t="str">
+        <v/>
+      </c>
       <c r="J52" t="str">
         <v>川菜</v>
       </c>
@@ -4819,6 +5215,12 @@
       <c r="G53" t="str">
         <v>亚坤YaKun餐厅(机场T3A店)</v>
       </c>
+      <c r="H53" t="str">
+        <v/>
+      </c>
+      <c r="I53" t="str">
+        <v/>
+      </c>
       <c r="J53" t="str">
         <v>东南亚菜</v>
       </c>
@@ -4905,6 +5307,12 @@
       <c r="G54" t="str">
         <v>熨斗糕老烧饼</v>
       </c>
+      <c r="H54" t="str">
+        <v/>
+      </c>
+      <c r="I54" t="str">
+        <v/>
+      </c>
       <c r="J54" t="str">
         <v>糕点</v>
       </c>
@@ -4991,6 +5399,12 @@
       <c r="G55" t="str">
         <v>茶颜悦色(PARK108国泰优活城市广场店)</v>
       </c>
+      <c r="H55" t="str">
+        <v/>
+      </c>
+      <c r="I55" t="str">
+        <v/>
+      </c>
       <c r="J55" t="str">
         <v>奶茶</v>
       </c>
@@ -5077,6 +5491,12 @@
       <c r="G56" t="str">
         <v>三样子(解放碑店)</v>
       </c>
+      <c r="H56" t="str">
+        <v/>
+      </c>
+      <c r="I56" t="str">
+        <v/>
+      </c>
       <c r="J56" t="str">
         <v>甜品</v>
       </c>
@@ -5163,6 +5583,12 @@
       <c r="G57" t="str">
         <v>李若桃·手作酸奶铺(解放碑八一路好吃街店)</v>
       </c>
+      <c r="H57" t="str">
+        <v/>
+      </c>
+      <c r="I57" t="str">
+        <v/>
+      </c>
       <c r="J57" t="str">
         <v>奶茶</v>
       </c>
@@ -5249,6 +5675,12 @@
       <c r="G58" t="str">
         <v>李氏串烧·鲜肉烧烤·江湖菜(巴南店)</v>
       </c>
+      <c r="H58" t="str">
+        <v/>
+      </c>
+      <c r="I58" t="str">
+        <v/>
+      </c>
       <c r="J58" t="str">
         <v>烧烤</v>
       </c>
@@ -5335,8 +5767,14 @@
       <c r="G59" t="str">
         <v>怪鸡脚(大坪店)</v>
       </c>
+      <c r="H59" t="str">
+        <v/>
+      </c>
+      <c r="I59" t="str">
+        <v/>
+      </c>
       <c r="J59" t="str">
-        <v>小吃</v>
+        <v>街头小吃</v>
       </c>
       <c r="K59" t="str">
         <v>street-food</v>
@@ -5397,6 +5835,9 @@
       </c>
       <c r="AD59" t="str">
         <v>branch</v>
+      </c>
+      <c r="AE59" t="str">
+        <v>街头小吃</v>
       </c>
     </row>
     <row r="60">
@@ -5421,6 +5862,12 @@
       <c r="G60" t="str">
         <v>朱富贵火锅(恒力城店)</v>
       </c>
+      <c r="H60" t="str">
+        <v/>
+      </c>
+      <c r="I60" t="str">
+        <v/>
+      </c>
       <c r="J60" t="str">
         <v>火锅</v>
       </c>
@@ -5507,6 +5954,12 @@
       <c r="G61" t="str">
         <v>肥婆肥仔海鲜档(平潭店)</v>
       </c>
+      <c r="H61" t="str">
+        <v/>
+      </c>
+      <c r="I61" t="str">
+        <v/>
+      </c>
       <c r="J61" t="str">
         <v>海鲜</v>
       </c>
@@ -5593,6 +6046,12 @@
       <c r="G62" t="str">
         <v>老朝凤水煮鱼(平潭店)</v>
       </c>
+      <c r="H62" t="str">
+        <v/>
+      </c>
+      <c r="I62" t="str">
+        <v/>
+      </c>
       <c r="J62" t="str">
         <v>火锅</v>
       </c>
@@ -5679,6 +6138,12 @@
       <c r="G63" t="str">
         <v>饼夫人</v>
       </c>
+      <c r="H63" t="str">
+        <v/>
+      </c>
+      <c r="I63" t="str">
+        <v/>
+      </c>
       <c r="J63" t="str">
         <v>糕点</v>
       </c>
@@ -5707,7 +6172,7 @@
         <v>周一至周日 08:30-23:00</v>
       </c>
       <c r="S63" t="str">
-        <v>13559610800;15960052072</v>
+        <v>13559610800；15960052072</v>
       </c>
       <c r="T63" t="str">
         <v>amap</v>
@@ -5765,8 +6230,14 @@
       <c r="G64" t="str">
         <v>煎意浓·吴记煎包(交通路店)</v>
       </c>
+      <c r="H64" t="str">
+        <v/>
+      </c>
+      <c r="I64" t="str">
+        <v/>
+      </c>
       <c r="J64" t="str">
-        <v>小吃</v>
+        <v>街头小吃</v>
       </c>
       <c r="K64" t="str">
         <v>street-food</v>
@@ -5827,6 +6298,9 @@
       </c>
       <c r="AD64" t="str">
         <v>branch</v>
+      </c>
+      <c r="AE64" t="str">
+        <v>街头小吃</v>
       </c>
     </row>
     <row r="65">
@@ -5851,8 +6325,14 @@
       <c r="G65" t="str">
         <v>福屿捞化(广达店)</v>
       </c>
+      <c r="H65" t="str">
+        <v/>
+      </c>
+      <c r="I65" t="str">
+        <v/>
+      </c>
       <c r="J65" t="str">
-        <v>小吃</v>
+        <v>街头小吃</v>
       </c>
       <c r="K65" t="str">
         <v>street-food</v>
@@ -5913,6 +6393,9 @@
       </c>
       <c r="AD65" t="str">
         <v>branch</v>
+      </c>
+      <c r="AE65" t="str">
+        <v>街头小吃</v>
       </c>
     </row>
     <row r="66">
@@ -5937,6 +6420,12 @@
       <c r="G66" t="str">
         <v>崔酱炸鸡(世欧广场店)</v>
       </c>
+      <c r="H66" t="str">
+        <v/>
+      </c>
+      <c r="I66" t="str">
+        <v/>
+      </c>
       <c r="J66" t="str">
         <v>快餐</v>
       </c>
@@ -6023,6 +6512,12 @@
       <c r="G67" t="str">
         <v>唐沫茶兮(东百中心C馆1楼店)</v>
       </c>
+      <c r="H67" t="str">
+        <v/>
+      </c>
+      <c r="I67" t="str">
+        <v/>
+      </c>
       <c r="J67" t="str">
         <v>奶茶</v>
       </c>
@@ -6109,8 +6604,14 @@
       <c r="G68" t="str">
         <v>叶叔醋肉</v>
       </c>
+      <c r="H68" t="str">
+        <v/>
+      </c>
+      <c r="I68" t="str">
+        <v/>
+      </c>
       <c r="J68" t="str">
-        <v>小吃</v>
+        <v>街头小吃</v>
       </c>
       <c r="K68" t="str">
         <v>street-food</v>
@@ -6171,6 +6672,9 @@
       </c>
       <c r="AD68" t="str">
         <v>branch</v>
+      </c>
+      <c r="AE68" t="str">
+        <v>街头小吃</v>
       </c>
     </row>
     <row r="69">
@@ -6195,6 +6699,12 @@
       <c r="G69" t="str">
         <v>谢记美食四果汤(六中店)</v>
       </c>
+      <c r="H69" t="str">
+        <v/>
+      </c>
+      <c r="I69" t="str">
+        <v/>
+      </c>
       <c r="J69" t="str">
         <v>甜品</v>
       </c>
@@ -6281,6 +6791,12 @@
       <c r="G70" t="str">
         <v>莓超疯(天台1店)</v>
       </c>
+      <c r="H70" t="str">
+        <v/>
+      </c>
+      <c r="I70" t="str">
+        <v/>
+      </c>
       <c r="J70" t="str">
         <v>奶茶</v>
       </c>
@@ -6367,8 +6883,14 @@
       <c r="G71" t="str">
         <v>东街钟楼肉粽(东街分店)</v>
       </c>
+      <c r="H71" t="str">
+        <v/>
+      </c>
+      <c r="I71" t="str">
+        <v/>
+      </c>
       <c r="J71" t="str">
-        <v>小吃</v>
+        <v>街头小吃</v>
       </c>
       <c r="K71" t="str">
         <v>street-food</v>
@@ -6395,7 +6917,7 @@
         <v>周一至周日 07:30-23:00</v>
       </c>
       <c r="S71" t="str">
-        <v>0595-22270165;0595-22952389;15060626033</v>
+        <v>0595-22270165；0595-22952389；15060626033</v>
       </c>
       <c r="T71" t="str">
         <v>amap</v>
@@ -6429,6 +6951,9 @@
       </c>
       <c r="AD71" t="str">
         <v>branch</v>
+      </c>
+      <c r="AE71" t="str">
+        <v>街头小吃</v>
       </c>
     </row>
     <row r="72">
@@ -6453,6 +6978,12 @@
       <c r="G72" t="str">
         <v>黄祥发牛排美食店(西湖店)</v>
       </c>
+      <c r="H72" t="str">
+        <v/>
+      </c>
+      <c r="I72" t="str">
+        <v/>
+      </c>
       <c r="J72" t="str">
         <v>牛排</v>
       </c>
@@ -6539,6 +7070,12 @@
       <c r="G73" t="str">
         <v>泮宫卤面(新门街店)</v>
       </c>
+      <c r="H73" t="str">
+        <v/>
+      </c>
+      <c r="I73" t="str">
+        <v/>
+      </c>
       <c r="J73" t="str">
         <v>面条</v>
       </c>
@@ -6625,6 +7162,12 @@
       <c r="G74" t="str">
         <v>水门国仔面线糊</v>
       </c>
+      <c r="H74" t="str">
+        <v/>
+      </c>
+      <c r="I74" t="str">
+        <v/>
+      </c>
       <c r="J74" t="str">
         <v>面条</v>
       </c>
@@ -6653,7 +7196,7 @@
         <v>周一至周日 00:00-24:00</v>
       </c>
       <c r="S74" t="str">
-        <v>15059548081;15305036963</v>
+        <v>15059548081；15305036963</v>
       </c>
       <c r="T74" t="str">
         <v>amap</v>
@@ -6711,6 +7254,12 @@
       <c r="G75" t="str">
         <v>肉食饭堂</v>
       </c>
+      <c r="H75" t="str">
+        <v/>
+      </c>
+      <c r="I75" t="str">
+        <v/>
+      </c>
       <c r="J75" t="str">
         <v>日料</v>
       </c>
@@ -6797,6 +7346,12 @@
       <c r="G76" t="str">
         <v>林锦记沙茶面(中山路步行街店)</v>
       </c>
+      <c r="H76" t="str">
+        <v/>
+      </c>
+      <c r="I76" t="str">
+        <v/>
+      </c>
       <c r="J76" t="str">
         <v>面条</v>
       </c>
@@ -6825,7 +7380,7 @@
         <v>周一至周日 08:00-23:00</v>
       </c>
       <c r="S76" t="str">
-        <v>18106088278;18396286852</v>
+        <v>18106088278；18396286852</v>
       </c>
       <c r="T76" t="str">
         <v>amap</v>
@@ -6883,6 +7438,12 @@
       <c r="G77" t="str">
         <v>壶见(中华城店)</v>
       </c>
+      <c r="H77" t="str">
+        <v/>
+      </c>
+      <c r="I77" t="str">
+        <v/>
+      </c>
       <c r="J77" t="str">
         <v>奶茶</v>
       </c>
@@ -6969,6 +7530,12 @@
       <c r="G78" t="str">
         <v>Juicy Bakery(大学路店)</v>
       </c>
+      <c r="H78" t="str">
+        <v/>
+      </c>
+      <c r="I78" t="str">
+        <v/>
+      </c>
       <c r="J78" t="str">
         <v>面包</v>
       </c>
@@ -7055,6 +7622,12 @@
       <c r="G79" t="str">
         <v>龚印记炭炉牛骨牛杂煲(珠影·星光城店)</v>
       </c>
+      <c r="H79" t="str">
+        <v/>
+      </c>
+      <c r="I79" t="str">
+        <v/>
+      </c>
       <c r="J79" t="str">
         <v>火锅</v>
       </c>
@@ -7141,6 +7714,12 @@
       <c r="G80" t="str">
         <v>陶陶居酒家(北京路店)</v>
       </c>
+      <c r="H80" t="str">
+        <v/>
+      </c>
+      <c r="I80" t="str">
+        <v/>
+      </c>
       <c r="J80" t="str">
         <v>粤菜</v>
       </c>
@@ -7169,7 +7748,7 @@
         <v>周一至周日 09:00-16:30，17:00-21:30</v>
       </c>
       <c r="S80" t="str">
-        <v>020-83700611;020-83700622</v>
+        <v>020-83700611；020-83700622</v>
       </c>
       <c r="T80" t="str">
         <v>amap</v>
@@ -7227,6 +7806,12 @@
       <c r="G81" t="str">
         <v>点都德(聚福楼)</v>
       </c>
+      <c r="H81" t="str">
+        <v/>
+      </c>
+      <c r="I81" t="str">
+        <v/>
+      </c>
       <c r="J81" t="str">
         <v>粤菜</v>
       </c>
@@ -7255,7 +7840,7 @@
         <v>周一至周日 08:00-16:00，17:00-21:00</v>
       </c>
       <c r="S81" t="str">
-        <v>13632423292;4001382828</v>
+        <v>13632423292；4001382828</v>
       </c>
       <c r="T81" t="str">
         <v>amap</v>
@@ -7313,6 +7898,12 @@
       <c r="G82" t="str">
         <v>银灯食府(文化公园店)</v>
       </c>
+      <c r="H82" t="str">
+        <v/>
+      </c>
+      <c r="I82" t="str">
+        <v/>
+      </c>
       <c r="J82" t="str">
         <v>粤菜</v>
       </c>
@@ -7399,6 +7990,12 @@
       <c r="G83" t="str">
         <v>潮发潮汕牛肉店(永庆坊店)</v>
       </c>
+      <c r="H83" t="str">
+        <v/>
+      </c>
+      <c r="I83" t="str">
+        <v/>
+      </c>
       <c r="J83" t="str">
         <v>火锅</v>
       </c>
@@ -7485,6 +8082,12 @@
       <c r="G84" t="str">
         <v>南信牛奶甜品专家</v>
       </c>
+      <c r="H84" t="str">
+        <v/>
+      </c>
+      <c r="I84" t="str">
+        <v/>
+      </c>
       <c r="J84" t="str">
         <v>甜品</v>
       </c>
@@ -7571,6 +8174,12 @@
       <c r="G85" t="str">
         <v>Paper Stone Bakery(北京路天河城店)</v>
       </c>
+      <c r="H85" t="str">
+        <v/>
+      </c>
+      <c r="I85" t="str">
+        <v/>
+      </c>
       <c r="J85" t="str">
         <v>面包</v>
       </c>
@@ -7657,6 +8266,12 @@
       <c r="G86" t="str">
         <v>双合园·海鲜水饺青岛菜(湛山店)</v>
       </c>
+      <c r="H86" t="str">
+        <v/>
+      </c>
+      <c r="I86" t="str">
+        <v/>
+      </c>
       <c r="J86" t="str">
         <v>海鲜</v>
       </c>
@@ -7743,6 +8358,12 @@
       <c r="G87" t="str">
         <v>华春餐馆</v>
       </c>
+      <c r="H87" t="str">
+        <v/>
+      </c>
+      <c r="I87" t="str">
+        <v/>
+      </c>
       <c r="J87" t="str">
         <v>海鲜</v>
       </c>
@@ -7771,7 +8392,7 @@
         <v>周一至周日 10:30-14:00，16:00-20:30</v>
       </c>
       <c r="S87" t="str">
-        <v>0532-82867990;0532-82882381</v>
+        <v>0532-82867990；0532-82882381</v>
       </c>
       <c r="T87" t="str">
         <v>amap</v>
@@ -7829,6 +8450,12 @@
       <c r="G88" t="str">
         <v>海乐海鲜家常菜</v>
       </c>
+      <c r="H88" t="str">
+        <v/>
+      </c>
+      <c r="I88" t="str">
+        <v/>
+      </c>
       <c r="J88" t="str">
         <v>海鲜</v>
       </c>
@@ -7915,6 +8542,12 @@
       <c r="G89" t="str">
         <v>新罗参鸡汤(市南麦凯乐店)</v>
       </c>
+      <c r="H89" t="str">
+        <v/>
+      </c>
+      <c r="I89" t="str">
+        <v/>
+      </c>
       <c r="J89" t="str">
         <v>韩餐</v>
       </c>
@@ -8001,6 +8634,12 @@
       <c r="G90" t="str">
         <v>August House八月小馆(鲁迅公园店)</v>
       </c>
+      <c r="H90" t="str">
+        <v/>
+      </c>
+      <c r="I90" t="str">
+        <v/>
+      </c>
       <c r="J90" t="str">
         <v>咖啡</v>
       </c>
@@ -8087,6 +8726,12 @@
       <c r="G91" t="str">
         <v>青岛王哥庄大馒头有限公司</v>
       </c>
+      <c r="H91" t="str">
+        <v/>
+      </c>
+      <c r="I91" t="str">
+        <v/>
+      </c>
       <c r="J91" t="str">
         <v>糕点</v>
       </c>
@@ -8101,6 +8746,9 @@
       </c>
       <c r="N91">
         <v>36.239358</v>
+      </c>
+      <c r="O91" t="str">
+        <v/>
       </c>
       <c r="P91">
         <v>1</v>
@@ -8170,6 +8818,12 @@
       <c r="G92" t="str">
         <v>小宫面包研究所(总部店)</v>
       </c>
+      <c r="H92" t="str">
+        <v/>
+      </c>
+      <c r="I92" t="str">
+        <v/>
+      </c>
       <c r="J92" t="str">
         <v>面包</v>
       </c>
@@ -8256,6 +8910,12 @@
       <c r="G93" t="str">
         <v>西园寺素食-面条</v>
       </c>
+      <c r="H93" t="str">
+        <v/>
+      </c>
+      <c r="I93" t="str">
+        <v/>
+      </c>
       <c r="J93" t="str">
         <v>面条</v>
       </c>
@@ -8342,6 +9002,12 @@
       <c r="G94" t="str">
         <v>裕兴记苏式汤面(星斓荟·路劲广场店)</v>
       </c>
+      <c r="H94" t="str">
+        <v/>
+      </c>
+      <c r="I94" t="str">
+        <v/>
+      </c>
       <c r="J94" t="str">
         <v>面条</v>
       </c>
@@ -8428,6 +9094,12 @@
       <c r="G95" t="str">
         <v>大孃孃糖水铺(双塔市集店)</v>
       </c>
+      <c r="H95" t="str">
+        <v/>
+      </c>
+      <c r="I95" t="str">
+        <v/>
+      </c>
       <c r="J95" t="str">
         <v>甜品</v>
       </c>
@@ -8512,7 +9184,13 @@
         <v>lstmg</v>
       </c>
       <c r="G96" t="str">
-        <v>老石头面条</v>
+        <v>老石头面馆</v>
+      </c>
+      <c r="H96" t="str">
+        <v/>
+      </c>
+      <c r="I96" t="str">
+        <v/>
       </c>
       <c r="J96" t="str">
         <v>面条</v>
@@ -8600,6 +9278,12 @@
       <c r="G97" t="str">
         <v>梅月轩·梅花糕(平江路店)</v>
       </c>
+      <c r="H97" t="str">
+        <v/>
+      </c>
+      <c r="I97" t="str">
+        <v/>
+      </c>
       <c r="J97" t="str">
         <v>糕点</v>
       </c>
@@ -8686,6 +9370,12 @@
       <c r="G98" t="str">
         <v>茉香枕河(平江路一店)</v>
       </c>
+      <c r="H98" t="str">
+        <v/>
+      </c>
+      <c r="I98" t="str">
+        <v/>
+      </c>
       <c r="J98" t="str">
         <v>冰淇淋</v>
       </c>
@@ -8772,6 +9462,12 @@
       <c r="G99" t="str">
         <v>稻香村(观前街店)</v>
       </c>
+      <c r="H99" t="str">
+        <v/>
+      </c>
+      <c r="I99" t="str">
+        <v/>
+      </c>
       <c r="J99" t="str">
         <v>糕点</v>
       </c>
@@ -8858,6 +9554,12 @@
       <c r="G100" t="str">
         <v>BONJOUR本就(苏州十全街店)</v>
       </c>
+      <c r="H100" t="str">
+        <v/>
+      </c>
+      <c r="I100" t="str">
+        <v/>
+      </c>
       <c r="J100" t="str">
         <v>奶茶</v>
       </c>
@@ -8944,8 +9646,14 @@
       <c r="G101" t="str">
         <v>朱新年点心店(山塘街店)</v>
       </c>
+      <c r="H101" t="str">
+        <v/>
+      </c>
+      <c r="I101" t="str">
+        <v/>
+      </c>
       <c r="J101" t="str">
-        <v>小吃</v>
+        <v>街头小吃</v>
       </c>
       <c r="K101" t="str">
         <v>street-food</v>
@@ -9006,6 +9714,9 @@
       </c>
       <c r="AD101" t="str">
         <v>branch</v>
+      </c>
+      <c r="AE101" t="str">
+        <v>街头小吃</v>
       </c>
     </row>
     <row r="102">
@@ -9030,8 +9741,14 @@
       <c r="G102" t="str">
         <v>鑫震源·苏式大虾生煎(人民路店)</v>
       </c>
+      <c r="H102" t="str">
+        <v/>
+      </c>
+      <c r="I102" t="str">
+        <v/>
+      </c>
       <c r="J102" t="str">
-        <v>小吃</v>
+        <v>街头小吃</v>
       </c>
       <c r="K102" t="str">
         <v>street-food</v>
@@ -9092,6 +9809,9 @@
       </c>
       <c r="AD102" t="str">
         <v>branch</v>
+      </c>
+      <c r="AE102" t="str">
+        <v>街头小吃</v>
       </c>
     </row>
     <row r="103">
@@ -9116,6 +9836,12 @@
       <c r="G103" t="str">
         <v>一乐韩国炸鸡(苏州店)</v>
       </c>
+      <c r="H103" t="str">
+        <v/>
+      </c>
+      <c r="I103" t="str">
+        <v/>
+      </c>
       <c r="J103" t="str">
         <v>快餐</v>
       </c>
@@ -9202,6 +9928,12 @@
       <c r="G104" t="str">
         <v>东海咖啡馆</v>
       </c>
+      <c r="H104" t="str">
+        <v/>
+      </c>
+      <c r="I104" t="str">
+        <v/>
+      </c>
       <c r="J104" t="str">
         <v>咖啡</v>
       </c>
@@ -9288,6 +10020,12 @@
       <c r="G105" t="str">
         <v>潘小烧·云南烧烤(外滩店)</v>
       </c>
+      <c r="H105" t="str">
+        <v/>
+      </c>
+      <c r="I105" t="str">
+        <v/>
+      </c>
       <c r="J105" t="str">
         <v>烧烤</v>
       </c>
@@ -9374,6 +10112,12 @@
       <c r="G106" t="str">
         <v>OTF加州餐厅(上海人广来福士店)</v>
       </c>
+      <c r="H106" t="str">
+        <v/>
+      </c>
+      <c r="I106" t="str">
+        <v/>
+      </c>
       <c r="J106" t="str">
         <v>西餐</v>
       </c>
@@ -9460,6 +10204,12 @@
       <c r="G107" t="str">
         <v>Bco豆库(CP静安店)</v>
       </c>
+      <c r="H107" t="str">
+        <v/>
+      </c>
+      <c r="I107" t="str">
+        <v/>
+      </c>
       <c r="J107" t="str">
         <v>融合菜</v>
       </c>
@@ -9546,6 +10296,12 @@
       <c r="G108" t="str">
         <v>3号仓库·创意中国菜(五角场店)</v>
       </c>
+      <c r="H108" t="str">
+        <v/>
+      </c>
+      <c r="I108" t="str">
+        <v/>
+      </c>
       <c r="J108" t="str">
         <v>融合菜</v>
       </c>
@@ -9632,6 +10388,12 @@
       <c r="G109" t="str">
         <v>米仓食堂(巴黎春天淮海V店店)</v>
       </c>
+      <c r="H109" t="str">
+        <v/>
+      </c>
+      <c r="I109" t="str">
+        <v/>
+      </c>
       <c r="J109" t="str">
         <v>融合菜</v>
       </c>
@@ -9718,6 +10480,12 @@
       <c r="G110" t="str">
         <v>MINI RESTAURANT小餐馆</v>
       </c>
+      <c r="H110" t="str">
+        <v/>
+      </c>
+      <c r="I110" t="str">
+        <v/>
+      </c>
       <c r="J110" t="str">
         <v>融合菜</v>
       </c>
@@ -9804,6 +10572,12 @@
       <c r="G111" t="str">
         <v>大馥·炭火烧肉酒场(梅川路店)</v>
       </c>
+      <c r="H111" t="str">
+        <v/>
+      </c>
+      <c r="I111" t="str">
+        <v/>
+      </c>
       <c r="J111" t="str">
         <v>烤肉</v>
       </c>
@@ -9890,6 +10664,12 @@
       <c r="G112" t="str">
         <v>锅气·湖南饭店(徐汇万科店)</v>
       </c>
+      <c r="H112" t="str">
+        <v/>
+      </c>
+      <c r="I112" t="str">
+        <v/>
+      </c>
       <c r="J112" t="str">
         <v>湘菜</v>
       </c>
@@ -9976,6 +10756,12 @@
       <c r="G113" t="str">
         <v>PINTXOS 西班牙小馆(国金中心店)</v>
       </c>
+      <c r="H113" t="str">
+        <v/>
+      </c>
+      <c r="I113" t="str">
+        <v/>
+      </c>
       <c r="J113" t="str">
         <v>西班牙菜</v>
       </c>
@@ -10004,7 +10790,7 @@
         <v>周一至周日 11:00-22:00</v>
       </c>
       <c r="S113" t="str">
-        <v>021-56752817;18466611561</v>
+        <v>021-56752817；18466611561</v>
       </c>
       <c r="T113" t="str">
         <v>amap</v>
@@ -10062,6 +10848,12 @@
       <c r="G114" t="str">
         <v>POETS泰狮(西岸梦中心店)</v>
       </c>
+      <c r="H114" t="str">
+        <v/>
+      </c>
+      <c r="I114" t="str">
+        <v/>
+      </c>
       <c r="J114" t="str">
         <v>东南亚菜</v>
       </c>
@@ -10148,6 +10940,12 @@
       <c r="G115" t="str">
         <v>耶里夏丽(田林东路店)</v>
       </c>
+      <c r="H115" t="str">
+        <v/>
+      </c>
+      <c r="I115" t="str">
+        <v/>
+      </c>
       <c r="J115" t="str">
         <v>新疆菜</v>
       </c>
@@ -10176,7 +10974,7 @@
         <v>周一至周日 10:00-22:00</v>
       </c>
       <c r="S115" t="str">
-        <v>021-64519797;19959006298</v>
+        <v>021-64519797；19959006298</v>
       </c>
       <c r="T115" t="str">
         <v>amap</v>
@@ -10234,6 +11032,12 @@
       <c r="G116" t="str">
         <v>耶里夏丽·新疆菜·西域宴(徐汇旗舰店)</v>
       </c>
+      <c r="H116" t="str">
+        <v/>
+      </c>
+      <c r="I116" t="str">
+        <v/>
+      </c>
       <c r="J116" t="str">
         <v>新疆菜</v>
       </c>
@@ -10320,6 +11124,12 @@
       <c r="G117" t="str">
         <v>今日牛事潮州牛肉火锅</v>
       </c>
+      <c r="H117" t="str">
+        <v/>
+      </c>
+      <c r="I117" t="str">
+        <v/>
+      </c>
       <c r="J117" t="str">
         <v>火锅</v>
       </c>
@@ -10406,6 +11216,12 @@
       <c r="G118" t="str">
         <v>手工红烧牛肉面大锅羊肉汤(安顺路231弄小区店)</v>
       </c>
+      <c r="H118" t="str">
+        <v/>
+      </c>
+      <c r="I118" t="str">
+        <v/>
+      </c>
       <c r="J118" t="str">
         <v>面条</v>
       </c>
@@ -10434,7 +11250,7 @@
         <v>周一至周日 00:00-24:00</v>
       </c>
       <c r="S118" t="str">
-        <v>13003292875;15000825010</v>
+        <v>13003292875；15000825010</v>
       </c>
       <c r="T118" t="str">
         <v>amap</v>
@@ -10492,6 +11308,12 @@
       <c r="G119" t="str">
         <v>哥哥の深夜食堂(正大乐城店)</v>
       </c>
+      <c r="H119" t="str">
+        <v/>
+      </c>
+      <c r="I119" t="str">
+        <v/>
+      </c>
       <c r="J119" t="str">
         <v>日料</v>
       </c>
@@ -10578,6 +11400,12 @@
       <c r="G120" t="str">
         <v>南里山房(上海来福士广场店)</v>
       </c>
+      <c r="H120" t="str">
+        <v/>
+      </c>
+      <c r="I120" t="str">
+        <v/>
+      </c>
       <c r="J120" t="str">
         <v>苏菜</v>
       </c>
@@ -10664,6 +11492,12 @@
       <c r="G121" t="str">
         <v>南里山房(上海荟聚店)</v>
       </c>
+      <c r="H121" t="str">
+        <v/>
+      </c>
+      <c r="I121" t="str">
+        <v/>
+      </c>
       <c r="J121" t="str">
         <v>苏菜</v>
       </c>
@@ -10750,6 +11584,12 @@
       <c r="G122" t="str">
         <v>井梅无锡私房面条</v>
       </c>
+      <c r="H122" t="str">
+        <v/>
+      </c>
+      <c r="I122" t="str">
+        <v/>
+      </c>
       <c r="J122" t="str">
         <v>苏菜</v>
       </c>
@@ -10836,6 +11676,12 @@
       <c r="G123" t="str">
         <v>香江姳苑(静安店)</v>
       </c>
+      <c r="H123" t="str">
+        <v/>
+      </c>
+      <c r="I123" t="str">
+        <v/>
+      </c>
       <c r="J123" t="str">
         <v>粤菜</v>
       </c>
@@ -10922,6 +11768,12 @@
       <c r="G124" t="str">
         <v>令谷花开·惊世料理(静安店)</v>
       </c>
+      <c r="H124" t="str">
+        <v/>
+      </c>
+      <c r="I124" t="str">
+        <v/>
+      </c>
       <c r="J124" t="str">
         <v>日料</v>
       </c>
@@ -10950,7 +11802,7 @@
         <v>周一至周日 11:00-22:30</v>
       </c>
       <c r="S124" t="str">
-        <v>021-63269030;13585705457</v>
+        <v>021-63269030；13585705457</v>
       </c>
       <c r="T124" t="str">
         <v>amap</v>
@@ -11008,6 +11860,12 @@
       <c r="G125" t="str">
         <v>强记發發牛肉汤</v>
       </c>
+      <c r="H125" t="str">
+        <v/>
+      </c>
+      <c r="I125" t="str">
+        <v/>
+      </c>
       <c r="J125" t="str">
         <v>面条</v>
       </c>
@@ -11094,6 +11952,12 @@
       <c r="G126" t="str">
         <v>猫十九·黑鱼花(品域·凌云里店)</v>
       </c>
+      <c r="H126" t="str">
+        <v/>
+      </c>
+      <c r="I126" t="str">
+        <v/>
+      </c>
       <c r="J126" t="str">
         <v>川菜</v>
       </c>
@@ -11180,6 +12044,12 @@
       <c r="G127" t="str">
         <v>浩海火烧云傣家菜(静安芮欧店)</v>
       </c>
+      <c r="H127" t="str">
+        <v/>
+      </c>
+      <c r="I127" t="str">
+        <v/>
+      </c>
       <c r="J127" t="str">
         <v>东南亚菜</v>
       </c>
@@ -11266,6 +12136,12 @@
       <c r="G128" t="str">
         <v>滇牛云南酸菜牛肉火锅(好又多上海田林分沃尔玛店)</v>
       </c>
+      <c r="H128" t="str">
+        <v/>
+      </c>
+      <c r="I128" t="str">
+        <v/>
+      </c>
       <c r="J128" t="str">
         <v>火锅</v>
       </c>
@@ -11352,6 +12228,12 @@
       <c r="G129" t="str">
         <v>裕兴记•蟹黄面条(上海首店)</v>
       </c>
+      <c r="H129" t="str">
+        <v/>
+      </c>
+      <c r="I129" t="str">
+        <v/>
+      </c>
       <c r="J129" t="str">
         <v>面条</v>
       </c>
@@ -11380,7 +12262,7 @@
         <v>周一至周日 08:00-20:00</v>
       </c>
       <c r="S129" t="str">
-        <v>13764519976;13917288228</v>
+        <v>13764519976；13917288228</v>
       </c>
       <c r="T129" t="str">
         <v>amap</v>
@@ -11438,6 +12320,12 @@
       <c r="G130" t="str">
         <v>湊湊火锅·茶憩(环贸iapm商场店)</v>
       </c>
+      <c r="H130" t="str">
+        <v/>
+      </c>
+      <c r="I130" t="str">
+        <v/>
+      </c>
       <c r="J130" t="str">
         <v>火锅</v>
       </c>
@@ -11466,7 +12354,7 @@
         <v>周一至周日 10:00-22:00</v>
       </c>
       <c r="S130" t="str">
-        <v>021-60700500;15261382830;15821431687</v>
+        <v>021-60700500；15261382830；15821431687</v>
       </c>
       <c r="T130" t="str">
         <v>amap</v>
@@ -11524,6 +12412,12 @@
       <c r="G131" t="str">
         <v>九老汉·川渝江湖菜(合川路店)</v>
       </c>
+      <c r="H131" t="str">
+        <v/>
+      </c>
+      <c r="I131" t="str">
+        <v/>
+      </c>
       <c r="J131" t="str">
         <v>川菜</v>
       </c>
@@ -11610,6 +12504,12 @@
       <c r="G132" t="str">
         <v>胖哥俩肉蟹煲(百联南桥购物中心店)</v>
       </c>
+      <c r="H132" t="str">
+        <v/>
+      </c>
+      <c r="I132" t="str">
+        <v/>
+      </c>
       <c r="J132" t="str">
         <v>海鲜</v>
       </c>
@@ -11696,6 +12596,12 @@
       <c r="G133" t="str">
         <v>萨莉亚意式餐厅(美乐源·华东理工站店)</v>
       </c>
+      <c r="H133" t="str">
+        <v/>
+      </c>
+      <c r="I133" t="str">
+        <v/>
+      </c>
       <c r="J133" t="str">
         <v>意大利菜</v>
       </c>
@@ -11782,6 +12688,12 @@
       <c r="G134" t="str">
         <v>粤潮馆(中兴路店)</v>
       </c>
+      <c r="H134" t="str">
+        <v/>
+      </c>
+      <c r="I134" t="str">
+        <v/>
+      </c>
       <c r="J134" t="str">
         <v>粤菜</v>
       </c>
@@ -11868,6 +12780,12 @@
       <c r="G135" t="str">
         <v>纪录片《人生一串》体验店(天山路店)</v>
       </c>
+      <c r="H135" t="str">
+        <v/>
+      </c>
+      <c r="I135" t="str">
+        <v/>
+      </c>
       <c r="J135" t="str">
         <v>烧烤</v>
       </c>
@@ -11896,7 +12814,7 @@
         <v>周一至周五 16:00-01:30 | 周六至周日 11:00-02:00</v>
       </c>
       <c r="S135" t="str">
-        <v>021-50829008;19101628027</v>
+        <v>021-50829008；19101628027</v>
       </c>
       <c r="T135" t="str">
         <v>amap</v>
@@ -11954,6 +12872,12 @@
       <c r="G136" t="str">
         <v>九鼎轩脆毛肚火锅(五角场店)</v>
       </c>
+      <c r="H136" t="str">
+        <v/>
+      </c>
+      <c r="I136" t="str">
+        <v/>
+      </c>
       <c r="J136" t="str">
         <v>火锅</v>
       </c>
@@ -12040,6 +12964,12 @@
       <c r="G137" t="str">
         <v>人生一串(海尚·生活广场店)</v>
       </c>
+      <c r="H137" t="str">
+        <v/>
+      </c>
+      <c r="I137" t="str">
+        <v/>
+      </c>
       <c r="J137" t="str">
         <v>烧烤</v>
       </c>
@@ -12126,6 +13056,12 @@
       <c r="G138" t="str">
         <v>东北铁锅炖(海思路店)</v>
       </c>
+      <c r="H138" t="str">
+        <v/>
+      </c>
+      <c r="I138" t="str">
+        <v/>
+      </c>
       <c r="J138" t="str">
         <v>东北菜</v>
       </c>
@@ -12212,6 +13148,12 @@
       <c r="G139" t="str">
         <v>东北老菜馆</v>
       </c>
+      <c r="H139" t="str">
+        <v/>
+      </c>
+      <c r="I139" t="str">
+        <v/>
+      </c>
       <c r="J139" t="str">
         <v>东北菜</v>
       </c>
@@ -12298,6 +13240,12 @@
       <c r="G140" t="str">
         <v>三石屋日料(海尚·生活广场店)</v>
       </c>
+      <c r="H140" t="str">
+        <v/>
+      </c>
+      <c r="I140" t="str">
+        <v/>
+      </c>
       <c r="J140" t="str">
         <v>日料</v>
       </c>
@@ -12326,7 +13274,7 @@
         <v>周一至周日 10:00-22:00</v>
       </c>
       <c r="S140" t="str">
-        <v>13916104206;15221637322</v>
+        <v>13916104206；15221637322</v>
       </c>
       <c r="T140" t="str">
         <v>amap</v>
@@ -12384,6 +13332,12 @@
       <c r="G141" t="str">
         <v>鱼酷活鱼烤鱼(上海莲花路lala station店)</v>
       </c>
+      <c r="H141" t="str">
+        <v/>
+      </c>
+      <c r="I141" t="str">
+        <v/>
+      </c>
       <c r="J141" t="str">
         <v>火锅</v>
       </c>
@@ -12470,6 +13424,12 @@
       <c r="G142" t="str">
         <v>太琼糟粕醋·海南百年传统火锅(上海首店)</v>
       </c>
+      <c r="H142" t="str">
+        <v/>
+      </c>
+      <c r="I142" t="str">
+        <v/>
+      </c>
       <c r="J142" t="str">
         <v>火锅</v>
       </c>
@@ -12556,6 +13516,12 @@
       <c r="G143" t="str">
         <v>米赫曼新疆餐厅</v>
       </c>
+      <c r="H143" t="str">
+        <v/>
+      </c>
+      <c r="I143" t="str">
+        <v/>
+      </c>
       <c r="J143" t="str">
         <v>新疆菜</v>
       </c>
@@ -12584,7 +13550,7 @@
         <v>周一至周日 11:00-24:00</v>
       </c>
       <c r="S143" t="str">
-        <v>021-64232270;13918063642</v>
+        <v>021-64232270；13918063642</v>
       </c>
       <c r="T143" t="str">
         <v>amap</v>
@@ -12642,6 +13608,12 @@
       <c r="G144" t="str">
         <v>吴老幺火锅(海湾店)</v>
       </c>
+      <c r="H144" t="str">
+        <v/>
+      </c>
+      <c r="I144" t="str">
+        <v/>
+      </c>
       <c r="J144" t="str">
         <v>火锅</v>
       </c>
@@ -12728,6 +13700,12 @@
       <c r="G145" t="str">
         <v>俄士厨房(正大广场店)</v>
       </c>
+      <c r="H145" t="str">
+        <v/>
+      </c>
+      <c r="I145" t="str">
+        <v/>
+      </c>
       <c r="J145" t="str">
         <v>俄国菜</v>
       </c>
@@ -12814,6 +13792,12 @@
       <c r="G146" t="str">
         <v>Black Salt·黑盐南亚西餐厅(打浦桥店)</v>
       </c>
+      <c r="H146" t="str">
+        <v/>
+      </c>
+      <c r="I146" t="str">
+        <v/>
+      </c>
       <c r="J146" t="str">
         <v>东南亚菜</v>
       </c>
@@ -12900,6 +13884,12 @@
       <c r="G147" t="str">
         <v>山石榴·贵州菜(丰盛里店)</v>
       </c>
+      <c r="H147" t="str">
+        <v/>
+      </c>
+      <c r="I147" t="str">
+        <v/>
+      </c>
       <c r="J147" t="str">
         <v>贵州菜</v>
       </c>
@@ -12986,6 +13976,12 @@
       <c r="G148" t="str">
         <v>山东饭店</v>
       </c>
+      <c r="H148" t="str">
+        <v/>
+      </c>
+      <c r="I148" t="str">
+        <v/>
+      </c>
       <c r="J148" t="str">
         <v>鲁菜</v>
       </c>
@@ -13072,6 +14068,12 @@
       <c r="G149" t="str">
         <v>沪西老弄堂面条(广东路店)</v>
       </c>
+      <c r="H149" t="str">
+        <v/>
+      </c>
+      <c r="I149" t="str">
+        <v/>
+      </c>
       <c r="J149" t="str">
         <v>面条</v>
       </c>
@@ -13158,6 +14160,12 @@
       <c r="G150" t="str">
         <v>龙华素斋</v>
       </c>
+      <c r="H150" t="str">
+        <v/>
+      </c>
+      <c r="I150" t="str">
+        <v/>
+      </c>
       <c r="J150" t="str">
         <v>面条</v>
       </c>
@@ -13244,6 +14252,12 @@
       <c r="G151" t="str">
         <v>毒蛇面条(人民广场店)</v>
       </c>
+      <c r="H151" t="str">
+        <v/>
+      </c>
+      <c r="I151" t="str">
+        <v/>
+      </c>
       <c r="J151" t="str">
         <v>面条</v>
       </c>
@@ -13330,6 +14344,12 @@
       <c r="G152" t="str">
         <v>牛New寿喜烧(长宁龙之梦店)</v>
       </c>
+      <c r="H152" t="str">
+        <v/>
+      </c>
+      <c r="I152" t="str">
+        <v/>
+      </c>
       <c r="J152" t="str">
         <v>火锅</v>
       </c>
@@ -13416,6 +14436,12 @@
       <c r="G153" t="str">
         <v>一绪に寿喜烧·和牛烫捞(龙华会店)</v>
       </c>
+      <c r="H153" t="str">
+        <v/>
+      </c>
+      <c r="I153" t="str">
+        <v/>
+      </c>
       <c r="J153" t="str">
         <v>火锅</v>
       </c>
@@ -13502,6 +14528,12 @@
       <c r="G154" t="str">
         <v>蜀谭记·盐帮川菜(田尚坊店)</v>
       </c>
+      <c r="H154" t="str">
+        <v/>
+      </c>
+      <c r="I154" t="str">
+        <v/>
+      </c>
       <c r="J154" t="str">
         <v>川菜</v>
       </c>
@@ -13588,6 +14620,12 @@
       <c r="G155" t="str">
         <v>肖四女乐山跷脚牛肉</v>
       </c>
+      <c r="H155" t="str">
+        <v/>
+      </c>
+      <c r="I155" t="str">
+        <v/>
+      </c>
       <c r="J155" t="str">
         <v>川菜</v>
       </c>
@@ -13674,6 +14712,12 @@
       <c r="G156" t="str">
         <v>首尔猪排(海湾科技园大楼店)</v>
       </c>
+      <c r="H156" t="str">
+        <v/>
+      </c>
+      <c r="I156" t="str">
+        <v/>
+      </c>
       <c r="J156" t="str">
         <v>韩餐</v>
       </c>
@@ -13760,6 +14804,12 @@
       <c r="G157" t="str">
         <v>佬鲜纪·鲜切鸡火锅(徐汇万科广场店)</v>
       </c>
+      <c r="H157" t="str">
+        <v/>
+      </c>
+      <c r="I157" t="str">
+        <v/>
+      </c>
       <c r="J157" t="str">
         <v>火锅</v>
       </c>
@@ -13846,6 +14896,12 @@
       <c r="G158" t="str">
         <v>平成屋(世博源店)</v>
       </c>
+      <c r="H158" t="str">
+        <v/>
+      </c>
+      <c r="I158" t="str">
+        <v/>
+      </c>
       <c r="J158" t="str">
         <v>日料</v>
       </c>
@@ -13932,6 +14988,12 @@
       <c r="G159" t="str">
         <v>噗噗满手抓饭(前滩店)</v>
       </c>
+      <c r="H159" t="str">
+        <v/>
+      </c>
+      <c r="I159" t="str">
+        <v/>
+      </c>
       <c r="J159" t="str">
         <v>新疆菜</v>
       </c>
@@ -14018,6 +15080,12 @@
       <c r="G160" t="str">
         <v>ZAFFERANO西班牙海鲜饭</v>
       </c>
+      <c r="H160" t="str">
+        <v/>
+      </c>
+      <c r="I160" t="str">
+        <v/>
+      </c>
       <c r="J160" t="str">
         <v>西班牙菜</v>
       </c>
@@ -14104,6 +15172,12 @@
       <c r="G161" t="str">
         <v>避风塘(徐汇万科广场店)</v>
       </c>
+      <c r="H161" t="str">
+        <v/>
+      </c>
+      <c r="I161" t="str">
+        <v/>
+      </c>
       <c r="J161" t="str">
         <v>粤菜</v>
       </c>
@@ -14190,6 +15264,12 @@
       <c r="G162" t="str">
         <v>蘩楼(淮海百盛店)</v>
       </c>
+      <c r="H162" t="str">
+        <v/>
+      </c>
+      <c r="I162" t="str">
+        <v/>
+      </c>
       <c r="J162" t="str">
         <v>粤菜</v>
       </c>
@@ -14276,6 +15356,12 @@
       <c r="G163" t="str">
         <v>上海迪士尼度假区</v>
       </c>
+      <c r="H163" t="str">
+        <v/>
+      </c>
+      <c r="I163" t="str">
+        <v/>
+      </c>
       <c r="J163" t="str">
         <v>快餐</v>
       </c>
@@ -14290,6 +15376,9 @@
       </c>
       <c r="N163">
         <v>31.141447</v>
+      </c>
+      <c r="O163" t="str">
+        <v/>
       </c>
       <c r="P163">
         <v>4.9</v>
@@ -14359,6 +15448,12 @@
       <c r="G164" t="str">
         <v>Money Shops(愚园路店)</v>
       </c>
+      <c r="H164" t="str">
+        <v/>
+      </c>
+      <c r="I164" t="str">
+        <v/>
+      </c>
       <c r="J164" t="str">
         <v>西餐</v>
       </c>
@@ -14445,6 +15540,12 @@
       <c r="G165" t="str">
         <v>Wagas沃歌斯(上海徐汇万科中心店)</v>
       </c>
+      <c r="H165" t="str">
+        <v/>
+      </c>
+      <c r="I165" t="str">
+        <v/>
+      </c>
       <c r="J165" t="str">
         <v>轻食</v>
       </c>
@@ -14531,6 +15632,12 @@
       <c r="G166" t="str">
         <v>baker&amp;spice(上海安福路店)</v>
       </c>
+      <c r="H166" t="str">
+        <v/>
+      </c>
+      <c r="I166" t="str">
+        <v/>
+      </c>
       <c r="J166" t="str">
         <v>轻食</v>
       </c>
@@ -14617,6 +15724,12 @@
       <c r="G167" t="str">
         <v>LOKAL东湖路店</v>
       </c>
+      <c r="H167" t="str">
+        <v/>
+      </c>
+      <c r="I167" t="str">
+        <v/>
+      </c>
       <c r="J167" t="str">
         <v>轻食</v>
       </c>
@@ -14703,6 +15816,12 @@
       <c r="G168" t="str">
         <v>gaga(上海环球港店)</v>
       </c>
+      <c r="H168" t="str">
+        <v/>
+      </c>
+      <c r="I168" t="str">
+        <v/>
+      </c>
       <c r="J168" t="str">
         <v>轻食</v>
       </c>
@@ -14789,6 +15908,12 @@
       <c r="G169" t="str">
         <v>Shake Shack(上海荟聚店)</v>
       </c>
+      <c r="H169" t="str">
+        <v/>
+      </c>
+      <c r="I169" t="str">
+        <v/>
+      </c>
       <c r="J169" t="str">
         <v>快餐</v>
       </c>
@@ -14875,6 +16000,12 @@
       <c r="G170" t="str">
         <v>Azabuya麻布屋(复兴西路洋房店)</v>
       </c>
+      <c r="H170" t="str">
+        <v/>
+      </c>
+      <c r="I170" t="str">
+        <v/>
+      </c>
       <c r="J170" t="str">
         <v>冰淇淋</v>
       </c>
@@ -14961,6 +16092,12 @@
       <c r="G171" t="str">
         <v>Luneurs(洛克·外滩源店)</v>
       </c>
+      <c r="H171" t="str">
+        <v/>
+      </c>
+      <c r="I171" t="str">
+        <v/>
+      </c>
       <c r="J171" t="str">
         <v>冰淇淋</v>
       </c>
@@ -15047,6 +16184,12 @@
       <c r="G172" t="str">
         <v>Mill Hill迷路之丘(吉宝静安中心店)</v>
       </c>
+      <c r="H172" t="str">
+        <v/>
+      </c>
+      <c r="I172" t="str">
+        <v/>
+      </c>
       <c r="J172" t="str">
         <v>咖啡</v>
       </c>
@@ -15133,6 +16276,12 @@
       <c r="G173" t="str">
         <v>Pns Cafe</v>
       </c>
+      <c r="H173" t="str">
+        <v/>
+      </c>
+      <c r="I173" t="str">
+        <v/>
+      </c>
       <c r="J173" t="str">
         <v>咖啡</v>
       </c>
@@ -15148,11 +16297,17 @@
       <c r="N173">
         <v>31.228357</v>
       </c>
+      <c r="O173" t="str">
+        <v/>
+      </c>
       <c r="P173">
         <v>4</v>
       </c>
       <c r="Q173" t="str">
         <v>CNY</v>
+      </c>
+      <c r="R173" t="str">
+        <v/>
       </c>
       <c r="S173" t="str">
         <v>[]</v>
@@ -15213,6 +16368,12 @@
       <c r="G174" t="str">
         <v>Hidden Track</v>
       </c>
+      <c r="H174" t="str">
+        <v/>
+      </c>
+      <c r="I174" t="str">
+        <v/>
+      </c>
       <c r="J174" t="str">
         <v>咖啡</v>
       </c>
@@ -15299,6 +16460,12 @@
       <c r="G175" t="str">
         <v>HILL CAFE</v>
       </c>
+      <c r="H175" t="str">
+        <v/>
+      </c>
+      <c r="I175" t="str">
+        <v/>
+      </c>
       <c r="J175" t="str">
         <v>咖啡</v>
       </c>
@@ -15385,6 +16552,12 @@
       <c r="G176" t="str">
         <v>Geographer地理学家咖啡(商场世纪汇广场店)</v>
       </c>
+      <c r="H176" t="str">
+        <v/>
+      </c>
+      <c r="I176" t="str">
+        <v/>
+      </c>
       <c r="J176" t="str">
         <v>咖啡</v>
       </c>
@@ -15471,6 +16644,12 @@
       <c r="G177" t="str">
         <v>9 ISLANDS(大宁858国际公寓店)</v>
       </c>
+      <c r="H177" t="str">
+        <v/>
+      </c>
+      <c r="I177" t="str">
+        <v/>
+      </c>
       <c r="J177" t="str">
         <v>酒吧</v>
       </c>
@@ -15557,6 +16736,12 @@
       <c r="G178" t="str">
         <v>PLUTO(龙华会店)</v>
       </c>
+      <c r="H178" t="str">
+        <v/>
+      </c>
+      <c r="I178" t="str">
+        <v/>
+      </c>
       <c r="J178" t="str">
         <v>酒吧</v>
       </c>
@@ -15643,6 +16828,12 @@
       <c r="G179" t="str">
         <v>Wooden Paradise木制天堂(长乐路店)</v>
       </c>
+      <c r="H179" t="str">
+        <v/>
+      </c>
+      <c r="I179" t="str">
+        <v/>
+      </c>
       <c r="J179" t="str">
         <v>酒吧</v>
       </c>
@@ -15729,6 +16920,12 @@
       <c r="G180" t="str">
         <v>KISS LAB</v>
       </c>
+      <c r="H180" t="str">
+        <v/>
+      </c>
+      <c r="I180" t="str">
+        <v/>
+      </c>
       <c r="J180" t="str">
         <v>酒吧</v>
       </c>
@@ -15815,6 +17012,12 @@
       <c r="G181" t="str">
         <v>仝TONIC BAR(CP静安店)</v>
       </c>
+      <c r="H181" t="str">
+        <v/>
+      </c>
+      <c r="I181" t="str">
+        <v/>
+      </c>
       <c r="J181" t="str">
         <v>酒吧</v>
       </c>
@@ -15901,6 +17104,12 @@
       <c r="G182" t="str">
         <v>鹅庄·台湾美食(古美路店)</v>
       </c>
+      <c r="H182" t="str">
+        <v/>
+      </c>
+      <c r="I182" t="str">
+        <v/>
+      </c>
       <c r="J182" t="str">
         <v>酒吧</v>
       </c>
@@ -15987,6 +17196,12 @@
       <c r="G183" t="str">
         <v>楚褚热干面(田林路店)</v>
       </c>
+      <c r="H183" t="str">
+        <v/>
+      </c>
+      <c r="I183" t="str">
+        <v/>
+      </c>
       <c r="J183" t="str">
         <v>酒吧</v>
       </c>
@@ -16073,6 +17288,12 @@
       <c r="G184" t="str">
         <v>胡麻(静安嘉里中心店)</v>
       </c>
+      <c r="H184" t="str">
+        <v/>
+      </c>
+      <c r="I184" t="str">
+        <v/>
+      </c>
       <c r="J184" t="str">
         <v>融合菜</v>
       </c>
@@ -16159,6 +17380,12 @@
       <c r="G185" t="str">
         <v>Blueglass酸奶(徐汇漕河泾印象城店)</v>
       </c>
+      <c r="H185" t="str">
+        <v/>
+      </c>
+      <c r="I185" t="str">
+        <v/>
+      </c>
       <c r="J185" t="str">
         <v>奶茶</v>
       </c>
@@ -16245,6 +17472,12 @@
       <c r="G186" t="str">
         <v>宝珠奶酪(徐汇漕河泾店)</v>
       </c>
+      <c r="H186" t="str">
+        <v/>
+      </c>
+      <c r="I186" t="str">
+        <v/>
+      </c>
       <c r="J186" t="str">
         <v>奶茶</v>
       </c>
@@ -16273,7 +17506,7 @@
         <v>周一至周日 10:00-21:00</v>
       </c>
       <c r="S186" t="str">
-        <v>13122190381;15201824622</v>
+        <v>13122190381；15201824622</v>
       </c>
       <c r="T186" t="str">
         <v>amap</v>
@@ -16331,6 +17564,12 @@
       <c r="G187" t="str">
         <v>太犇牛手作茶铺(静安寺玖博广场店)</v>
       </c>
+      <c r="H187" t="str">
+        <v/>
+      </c>
+      <c r="I187" t="str">
+        <v/>
+      </c>
       <c r="J187" t="str">
         <v>奶茶</v>
       </c>
@@ -16417,6 +17656,12 @@
       <c r="G188" t="str">
         <v>茉莉奶白(宝龙广场店)</v>
       </c>
+      <c r="H188" t="str">
+        <v/>
+      </c>
+      <c r="I188" t="str">
+        <v/>
+      </c>
       <c r="J188" t="str">
         <v>奶茶</v>
       </c>
@@ -16503,6 +17748,12 @@
       <c r="G189" t="str">
         <v>OT另茶(城市集市上海荟聚店)</v>
       </c>
+      <c r="H189" t="str">
+        <v/>
+      </c>
+      <c r="I189" t="str">
+        <v/>
+      </c>
       <c r="J189" t="str">
         <v>奶茶</v>
       </c>
@@ -16589,6 +17840,12 @@
       <c r="G190" t="str">
         <v>阿嬷手作(上海环贸iapm店)</v>
       </c>
+      <c r="H190" t="str">
+        <v/>
+      </c>
+      <c r="I190" t="str">
+        <v/>
+      </c>
       <c r="J190" t="str">
         <v>奶茶</v>
       </c>
@@ -16675,6 +17932,12 @@
       <c r="G191" t="str">
         <v>茶米有言(长宁龙之梦店)</v>
       </c>
+      <c r="H191" t="str">
+        <v/>
+      </c>
+      <c r="I191" t="str">
+        <v/>
+      </c>
       <c r="J191" t="str">
         <v>奶茶</v>
       </c>
@@ -16761,6 +18024,12 @@
       <c r="G192" t="str">
         <v>LAVAZZA拉瓦萨咖啡(上海徐汇万科店)</v>
       </c>
+      <c r="H192" t="str">
+        <v/>
+      </c>
+      <c r="I192" t="str">
+        <v/>
+      </c>
       <c r="J192" t="str">
         <v>咖啡</v>
       </c>
@@ -16847,6 +18116,12 @@
       <c r="G193" t="str">
         <v>石库制饼·现烤软曲奇</v>
       </c>
+      <c r="H193" t="str">
+        <v/>
+      </c>
+      <c r="I193" t="str">
+        <v/>
+      </c>
       <c r="J193" t="str">
         <v>甜品</v>
       </c>
@@ -16933,6 +18208,12 @@
       <c r="G194" t="str">
         <v>BASDBAN(愚园路餐厅)</v>
       </c>
+      <c r="H194" t="str">
+        <v/>
+      </c>
+      <c r="I194" t="str">
+        <v/>
+      </c>
       <c r="J194" t="str">
         <v>甜品</v>
       </c>
@@ -17019,6 +18300,12 @@
       <c r="G195" t="str">
         <v>brown sixty(天乐广场店)</v>
       </c>
+      <c r="H195" t="str">
+        <v/>
+      </c>
+      <c r="I195" t="str">
+        <v/>
+      </c>
       <c r="J195" t="str">
         <v>面包</v>
       </c>
@@ -17105,6 +18392,12 @@
       <c r="G196" t="str">
         <v>THE MATCHA TOKYO(前滩太古里店)</v>
       </c>
+      <c r="H196" t="str">
+        <v/>
+      </c>
+      <c r="I196" t="str">
+        <v/>
+      </c>
       <c r="J196" t="str">
         <v>奶茶</v>
       </c>
@@ -17191,6 +18484,12 @@
       <c r="G197" t="str">
         <v>读酥世家(徐汇万科广场)</v>
       </c>
+      <c r="H197" t="str">
+        <v/>
+      </c>
+      <c r="I197" t="str">
+        <v/>
+      </c>
       <c r="J197" t="str">
         <v>面包</v>
       </c>
@@ -17277,6 +18576,12 @@
       <c r="G198" t="str">
         <v>UH 祐禾(徐汇万科广场)</v>
       </c>
+      <c r="H198" t="str">
+        <v/>
+      </c>
+      <c r="I198" t="str">
+        <v/>
+      </c>
       <c r="J198" t="str">
         <v>面包</v>
       </c>
@@ -17363,6 +18668,12 @@
       <c r="G199" t="str">
         <v>BUTTER%(前滩陆家嘴店)</v>
       </c>
+      <c r="H199" t="str">
+        <v/>
+      </c>
+      <c r="I199" t="str">
+        <v/>
+      </c>
       <c r="J199" t="str">
         <v>甜品</v>
       </c>
@@ -17449,6 +18760,12 @@
       <c r="G200" t="str">
         <v>苹果花园(永德路步行街店)</v>
       </c>
+      <c r="H200" t="str">
+        <v/>
+      </c>
+      <c r="I200" t="str">
+        <v/>
+      </c>
       <c r="J200" t="str">
         <v>面包</v>
       </c>
@@ -17535,6 +18852,12 @@
       <c r="G201" t="str">
         <v>FASCINO BAKERY(幸福里店)</v>
       </c>
+      <c r="H201" t="str">
+        <v/>
+      </c>
+      <c r="I201" t="str">
+        <v/>
+      </c>
       <c r="J201" t="str">
         <v>面包</v>
       </c>
@@ -17621,6 +18944,12 @@
       <c r="G202" t="str">
         <v>WenTinG文汀半糖蛋糕(上海荟聚)</v>
       </c>
+      <c r="H202" t="str">
+        <v/>
+      </c>
+      <c r="I202" t="str">
+        <v/>
+      </c>
       <c r="J202" t="str">
         <v>甜品</v>
       </c>
@@ -17707,6 +19036,12 @@
       <c r="G203" t="str">
         <v>莉莲蛋挞(徐家汇中心店)</v>
       </c>
+      <c r="H203" t="str">
+        <v/>
+      </c>
+      <c r="I203" t="str">
+        <v/>
+      </c>
       <c r="J203" t="str">
         <v>面包</v>
       </c>
@@ -17793,6 +19128,12 @@
       <c r="G204" t="str">
         <v>HOTCRUSH趁热集合·现烤面包(美罗城店)</v>
       </c>
+      <c r="H204" t="str">
+        <v/>
+      </c>
+      <c r="I204" t="str">
+        <v/>
+      </c>
       <c r="J204" t="str">
         <v>面包</v>
       </c>
@@ -17879,6 +19220,12 @@
       <c r="G205" t="str">
         <v>BUTTERFUL&amp;CREAMOROUS(长宁龙之梦店)</v>
       </c>
+      <c r="H205" t="str">
+        <v/>
+      </c>
+      <c r="I205" t="str">
+        <v/>
+      </c>
       <c r="J205" t="str">
         <v>面包</v>
       </c>
@@ -17965,6 +19312,12 @@
       <c r="G206" t="str">
         <v>小方块甜点(新闸路店)</v>
       </c>
+      <c r="H206" t="str">
+        <v/>
+      </c>
+      <c r="I206" t="str">
+        <v/>
+      </c>
       <c r="J206" t="str">
         <v>甜品</v>
       </c>
@@ -17993,7 +19346,7 @@
         <v>周一至周日 11:30-21:30</v>
       </c>
       <c r="S206" t="str">
-        <v>15300660010;15921644331</v>
+        <v>15300660010；15921644331</v>
       </c>
       <c r="T206" t="str">
         <v>amap</v>
@@ -18051,6 +19404,12 @@
       <c r="G207" t="str">
         <v>DRUNK BAKER(田子坊店)</v>
       </c>
+      <c r="H207" t="str">
+        <v/>
+      </c>
+      <c r="I207" t="str">
+        <v/>
+      </c>
       <c r="J207" t="str">
         <v>甜品</v>
       </c>
@@ -18137,6 +19496,12 @@
       <c r="G208" t="str">
         <v>Punch Monday Bakery</v>
       </c>
+      <c r="H208" t="str">
+        <v/>
+      </c>
+      <c r="I208" t="str">
+        <v/>
+      </c>
       <c r="J208" t="str">
         <v>面包</v>
       </c>
@@ -18223,6 +19588,12 @@
       <c r="G209" t="str">
         <v>卡特司库(芮欧百货店)</v>
       </c>
+      <c r="H209" t="str">
+        <v/>
+      </c>
+      <c r="I209" t="str">
+        <v/>
+      </c>
       <c r="J209" t="str">
         <v>甜品</v>
       </c>
@@ -18309,6 +19680,12 @@
       <c r="G210" t="str">
         <v>虹口糕团食品厂(莘庄地铁站店)</v>
       </c>
+      <c r="H210" t="str">
+        <v/>
+      </c>
+      <c r="I210" t="str">
+        <v/>
+      </c>
       <c r="J210" t="str">
         <v>糕点</v>
       </c>
@@ -18395,6 +19772,12 @@
       <c r="G211" t="str">
         <v>上海哈尔滨食品厂</v>
       </c>
+      <c r="H211" t="str">
+        <v/>
+      </c>
+      <c r="I211" t="str">
+        <v/>
+      </c>
       <c r="J211" t="str">
         <v>面包</v>
       </c>
@@ -18481,6 +19864,12 @@
       <c r="G212" t="str">
         <v>ALDI奥乐齐(闵行银都海梦一方店)</v>
       </c>
+      <c r="H212" t="str">
+        <v/>
+      </c>
+      <c r="I212" t="str">
+        <v/>
+      </c>
       <c r="J212" t="str">
         <v>糕点</v>
       </c>
@@ -18495,6 +19884,9 @@
       </c>
       <c r="N212">
         <v>31.09958</v>
+      </c>
+      <c r="O212" t="str">
+        <v/>
       </c>
       <c r="P212">
         <v>4.5</v>
@@ -18564,8 +19956,14 @@
       <c r="G213" t="str">
         <v>华师大夜市</v>
       </c>
+      <c r="H213" t="str">
+        <v/>
+      </c>
+      <c r="I213" t="str">
+        <v/>
+      </c>
       <c r="J213" t="str">
-        <v>小吃</v>
+        <v>街头小吃</v>
       </c>
       <c r="K213" t="str">
         <v>street-food</v>
@@ -18626,6 +20024,9 @@
       </c>
       <c r="AD213" t="str">
         <v>branch</v>
+      </c>
+      <c r="AE213" t="str">
+        <v>街头小吃</v>
       </c>
     </row>
     <row r="214">
@@ -18650,8 +20051,14 @@
       <c r="G214" t="str">
         <v>黑暗料理街</v>
       </c>
+      <c r="H214" t="str">
+        <v/>
+      </c>
+      <c r="I214" t="str">
+        <v/>
+      </c>
       <c r="J214" t="str">
-        <v>小吃</v>
+        <v>街头小吃</v>
       </c>
       <c r="K214" t="str">
         <v>street-food</v>
@@ -18665,6 +20072,9 @@
       <c r="N214">
         <v>30.836653</v>
       </c>
+      <c r="O214" t="str">
+        <v/>
+      </c>
       <c r="P214">
         <v>4.2</v>
       </c>
@@ -18709,6 +20119,9 @@
       </c>
       <c r="AD214" t="str">
         <v>branch</v>
+      </c>
+      <c r="AE214" t="str">
+        <v>街头小吃</v>
       </c>
     </row>
     <row r="215">
@@ -18733,8 +20146,14 @@
       <c r="G215" t="str">
         <v>韩国美食一条街(井亭天地生活广场店)</v>
       </c>
+      <c r="H215" t="str">
+        <v/>
+      </c>
+      <c r="I215" t="str">
+        <v/>
+      </c>
       <c r="J215" t="str">
-        <v>小吃</v>
+        <v>街头小吃</v>
       </c>
       <c r="K215" t="str">
         <v>street-food</v>
@@ -18748,6 +20167,9 @@
       <c r="N215">
         <v>31.169963</v>
       </c>
+      <c r="O215" t="str">
+        <v/>
+      </c>
       <c r="P215">
         <v>4.7</v>
       </c>
@@ -18757,6 +20179,9 @@
       <c r="R215" t="str">
         <v>周一至周日 11:00-22:00</v>
       </c>
+      <c r="S215" t="str">
+        <v/>
+      </c>
       <c r="T215" t="str">
         <v>amap</v>
       </c>
@@ -18789,6 +20214,9 @@
       </c>
       <c r="AD215" t="str">
         <v>branch</v>
+      </c>
+      <c r="AE215" t="str">
+        <v>街头小吃</v>
       </c>
     </row>
     <row r="216">
@@ -18813,6 +20241,12 @@
       <c r="G216" t="str">
         <v>塘湾饮食店</v>
       </c>
+      <c r="H216" t="str">
+        <v/>
+      </c>
+      <c r="I216" t="str">
+        <v/>
+      </c>
       <c r="J216" t="str">
         <v>面馆</v>
       </c>
@@ -18899,6 +20333,12 @@
       <c r="G217" t="str">
         <v>台南肉燥饭(满天星生活广场店)</v>
       </c>
+      <c r="H217" t="str">
+        <v/>
+      </c>
+      <c r="I217" t="str">
+        <v/>
+      </c>
       <c r="J217" t="str">
         <v>快餐</v>
       </c>
@@ -18985,6 +20425,12 @@
       <c r="G218" t="str">
         <v>觅弄堂炸鸡(闵行店)</v>
       </c>
+      <c r="H218" t="str">
+        <v/>
+      </c>
+      <c r="I218" t="str">
+        <v/>
+      </c>
       <c r="J218" t="str">
         <v>快餐</v>
       </c>
@@ -19071,6 +20517,12 @@
       <c r="G219" t="str">
         <v>Guaka活力健康餐(前滩店)</v>
       </c>
+      <c r="H219" t="str">
+        <v/>
+      </c>
+      <c r="I219" t="str">
+        <v/>
+      </c>
       <c r="J219" t="str">
         <v>轻食</v>
       </c>
@@ -19099,7 +20551,7 @@
         <v>周一至周日 10:00-20:00</v>
       </c>
       <c r="S219" t="str">
-        <v>17321061364;19128794371</v>
+        <v>17321061364；19128794371</v>
       </c>
       <c r="T219" t="str">
         <v>amap</v>
@@ -19157,6 +20609,12 @@
       <c r="G220" t="str">
         <v>MISS POKE波奇海鲜饭(前滩店)</v>
       </c>
+      <c r="H220" t="str">
+        <v/>
+      </c>
+      <c r="I220" t="str">
+        <v/>
+      </c>
       <c r="J220" t="str">
         <v>轻食</v>
       </c>
@@ -19243,8 +20701,14 @@
       <c r="G221" t="str">
         <v>港式石磨肠粉潮汕原味汤粉王</v>
       </c>
+      <c r="H221" t="str">
+        <v/>
+      </c>
+      <c r="I221" t="str">
+        <v/>
+      </c>
       <c r="J221" t="str">
-        <v>小吃</v>
+        <v>街头小吃</v>
       </c>
       <c r="K221" t="str">
         <v>street-food</v>
@@ -19271,7 +20735,7 @@
         <v>周一至周日 07:30-23:20</v>
       </c>
       <c r="S221" t="str">
-        <v>18516147702;18850939210</v>
+        <v>18516147702；18850939210</v>
       </c>
       <c r="T221" t="str">
         <v>amap</v>
@@ -19305,6 +20769,9 @@
       </c>
       <c r="AD221" t="str">
         <v>branch</v>
+      </c>
+      <c r="AE221" t="str">
+        <v>街头小吃</v>
       </c>
     </row>
     <row r="222">
@@ -19329,8 +20796,14 @@
       <c r="G222" t="str">
         <v>彭浦一炸(永平路店)</v>
       </c>
+      <c r="H222" t="str">
+        <v/>
+      </c>
+      <c r="I222" t="str">
+        <v/>
+      </c>
       <c r="J222" t="str">
-        <v>小吃</v>
+        <v>街头小吃</v>
       </c>
       <c r="K222" t="str">
         <v>street-food</v>
@@ -19392,10 +20865,13 @@
       <c r="AD222" t="str">
         <v>brand</v>
       </c>
+      <c r="AE222" t="str">
+        <v>街头小吃</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD222"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AE222"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Shanghai stores and incremental R2 photo sync.
Expand 81bakery, mdmc, hzdc, drunk-baker, and related Shanghai photo/data entries; default photos:sync-r2 to git-based incremental upload with delete/rename support and update data-workflow docs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/src/data/restaurants.xlsx
+++ b/src/data/restaurants.xlsx
@@ -4,11 +4,14 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="28340" windowHeight="14120"/>
+    <workbookView windowWidth="29400" windowHeight="14120"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AF$291</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -27,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7107" uniqueCount="1781">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7197" uniqueCount="1800">
   <si>
     <t>city_zh</t>
   </si>
@@ -4926,6 +4929,63 @@
   </si>
   <si>
     <t>https://www.amap.com/place/B0JAXGVOKJ</t>
+  </si>
+  <si>
+    <t>hzdc</t>
+  </si>
+  <si>
+    <t>胡子大厨·超级小炒肉(传媒港G·WALK店)</t>
+  </si>
+  <si>
+    <t>龙文路199号传媒港G·WALK负一层B1-L区-11B(老乡鸡对面)</t>
+  </si>
+  <si>
+    <t>17737168579；19121401541</t>
+  </si>
+  <si>
+    <t>https://www.amap.com/place/B0LB7UOFE2</t>
+  </si>
+  <si>
+    <t>mdmc</t>
+  </si>
+  <si>
+    <t>抹岛抹茶MATCHA ISLAND(美罗城店)</t>
+  </si>
+  <si>
+    <t>MATCHA ISLAND</t>
+  </si>
+  <si>
+    <t>徐汇区肇嘉浜路1111号美罗城B1F层</t>
+  </si>
+  <si>
+    <t>https://www.amap.com/place/B0MAV56VRJ</t>
+  </si>
+  <si>
+    <t>DRUNK BAKER(西岸梦中心)</t>
+  </si>
+  <si>
+    <t>周五至周日 08:00-22:00 ｜ 周一至周四 10:00-22:00</t>
+  </si>
+  <si>
+    <t>13166225027</t>
+  </si>
+  <si>
+    <t>https://www.amap.com/place/B0K1GH032K</t>
+  </si>
+  <si>
+    <t>81bakery</t>
+  </si>
+  <si>
+    <t>81BAKERY(西岸梦中心店)</t>
+  </si>
+  <si>
+    <t>龙腾大道2260号西岸梦中心4栋4楼115号</t>
+  </si>
+  <si>
+    <t>19352158076</t>
+  </si>
+  <si>
+    <t>https://www.amap.com/place/B0L3O7Y26X</t>
   </si>
   <si>
     <t>苏州</t>
@@ -5845,154 +5905,153 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0">
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0">
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0">
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0">
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0">
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -6376,37 +6435,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AF287"/>
+  <dimension ref="A1:AF291"/>
   <sheetFormatPr defaultColWidth="9.64285714285714" defaultRowHeight="17.6"/>
   <cols>
-    <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="13.9285714285714" customWidth="1"/>
-    <col min="3" max="3" width="11.5" customWidth="1"/>
-    <col min="4" max="4" width="12.0714285714286" customWidth="1"/>
-    <col min="5" max="5" width="8.78571428571429" customWidth="1"/>
-    <col min="6" max="6" width="17.0714285714286" customWidth="1"/>
-    <col min="7" max="7" width="40.8839285714286" customWidth="1"/>
-    <col min="8" max="8" width="41.5" customWidth="1"/>
-    <col min="9" max="10" width="24" customWidth="1"/>
-    <col min="11" max="11" width="10.7857142857143" customWidth="1"/>
-    <col min="12" max="12" width="23.2142857142857" customWidth="1"/>
-    <col min="13" max="13" width="6.85714285714286" customWidth="1"/>
-    <col min="14" max="14" width="82.5446428571429" customWidth="1"/>
-    <col min="15" max="15" width="12.7857142857143" customWidth="1"/>
-    <col min="16" max="16" width="11.2142857142857" customWidth="1"/>
-    <col min="17" max="17" width="17.5" customWidth="1"/>
-    <col min="18" max="18" width="13.4285714285714" customWidth="1"/>
-    <col min="19" max="19" width="9" customWidth="1"/>
+    <col min="7" max="7" width="57.0714285714286" customWidth="1"/>
     <col min="20" max="20" width="109.928571428571" customWidth="1"/>
     <col min="21" max="21" width="45.9285714285714" customWidth="1"/>
-    <col min="23" max="23" width="223.857142857143" customWidth="1"/>
-    <col min="25" max="25" width="11.4285714285714" customWidth="1"/>
-    <col min="26" max="26" width="19.1428571428571" customWidth="1"/>
-    <col min="27" max="27" width="13.2857142857143" customWidth="1"/>
-    <col min="28" max="28" width="12.6428571428571" customWidth="1"/>
-    <col min="29" max="29" width="16.6428571428571" customWidth="1"/>
-    <col min="30" max="30" width="14.2857142857143" customWidth="1"/>
-    <col min="31" max="31" width="15.0714285714286" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:32">
@@ -8238,7 +8272,7 @@
       <c r="F21" t="s">
         <v>176</v>
       </c>
-      <c r="G21" s="1" t="s">
+      <c r="G21" t="s">
         <v>177</v>
       </c>
       <c r="H21" t="s">
@@ -30013,10 +30047,10 @@
     </row>
     <row r="264" spans="1:32">
       <c r="A264" t="s">
-        <v>1633</v>
+        <v>680</v>
       </c>
       <c r="B264" t="s">
-        <v>1634</v>
+        <v>681</v>
       </c>
       <c r="C264" t="s">
         <v>34</v>
@@ -30028,40 +30062,37 @@
         <v>36</v>
       </c>
       <c r="F264" t="s">
-        <v>1635</v>
+        <v>1633</v>
       </c>
       <c r="G264" t="s">
-        <v>1636</v>
-      </c>
-      <c r="H264" t="s">
-        <v>1637</v>
+        <v>1634</v>
       </c>
       <c r="J264" t="s">
         <v>53</v>
       </c>
       <c r="K264" t="s">
-        <v>66</v>
+        <v>996</v>
       </c>
       <c r="L264" t="s">
-        <v>67</v>
+        <v>997</v>
       </c>
       <c r="M264" t="s">
         <v>42</v>
       </c>
       <c r="N264" t="s">
-        <v>1638</v>
+        <v>1635</v>
       </c>
       <c r="O264">
-        <v>120.63475</v>
+        <v>121.462156</v>
       </c>
       <c r="P264">
-        <v>31.29909</v>
+        <v>31.159353</v>
       </c>
       <c r="Q264">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="R264">
-        <v>4.6</v>
+        <v>4.3</v>
       </c>
       <c r="S264" t="s">
         <v>44</v>
@@ -30070,28 +30101,28 @@
         <v>859</v>
       </c>
       <c r="U264" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="V264" t="s">
         <v>47</v>
       </c>
       <c r="W264" t="s">
-        <v>1640</v>
+        <v>1637</v>
       </c>
       <c r="X264" t="s">
-        <v>71</v>
-      </c>
-      <c r="Y264" t="s">
-        <v>52</v>
-      </c>
-      <c r="Z264" t="s">
-        <v>52</v>
-      </c>
-      <c r="AA264" t="s">
-        <v>52</v>
+        <v>49</v>
+      </c>
+      <c r="Y264">
+        <v>3</v>
+      </c>
+      <c r="Z264">
+        <v>3</v>
+      </c>
+      <c r="AA264">
+        <v>3</v>
       </c>
       <c r="AB264" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="AC264" t="s">
         <v>53</v>
@@ -30099,8 +30130,8 @@
       <c r="AD264" t="s">
         <v>53</v>
       </c>
-      <c r="AE264" t="s">
-        <v>52</v>
+      <c r="AE264">
+        <v>3</v>
       </c>
       <c r="AF264" t="s">
         <v>54</v>
@@ -30108,10 +30139,10 @@
     </row>
     <row r="265" spans="1:32">
       <c r="A265" t="s">
-        <v>1633</v>
+        <v>680</v>
       </c>
       <c r="B265" t="s">
-        <v>1634</v>
+        <v>681</v>
       </c>
       <c r="C265" t="s">
         <v>34</v>
@@ -30123,76 +30154,79 @@
         <v>36</v>
       </c>
       <c r="F265" t="s">
+        <v>1638</v>
+      </c>
+      <c r="G265" t="s">
+        <v>1639</v>
+      </c>
+      <c r="H265" t="s">
+        <v>1640</v>
+      </c>
+      <c r="J265" t="s">
+        <v>53</v>
+      </c>
+      <c r="K265" t="s">
+        <v>66</v>
+      </c>
+      <c r="L265" t="s">
+        <v>67</v>
+      </c>
+      <c r="M265" t="s">
+        <v>53</v>
+      </c>
+      <c r="N265" t="s">
         <v>1641</v>
       </c>
-      <c r="G265" t="s">
-        <v>1642</v>
-      </c>
-      <c r="J265" t="s">
-        <v>53</v>
-      </c>
-      <c r="K265" t="s">
-        <v>153</v>
-      </c>
-      <c r="L265" t="s">
-        <v>154</v>
-      </c>
-      <c r="M265" t="s">
-        <v>42</v>
-      </c>
-      <c r="N265" t="s">
-        <v>1643</v>
-      </c>
       <c r="O265">
-        <v>120.635604</v>
+        <v>121.439725</v>
       </c>
       <c r="P265">
-        <v>31.306522</v>
+        <v>31.193375</v>
       </c>
       <c r="Q265">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="R265">
-        <v>4.6</v>
+        <v>3.7</v>
       </c>
       <c r="S265" t="s">
         <v>44</v>
       </c>
       <c r="T265" t="s">
-        <v>1052</v>
-      </c>
-      <c r="U265" t="s">
-        <v>1644</v>
+        <v>744</v>
+      </c>
+      <c r="U265">
+        <v>17339617082</v>
       </c>
       <c r="V265" t="s">
         <v>47</v>
       </c>
       <c r="W265" t="s">
-        <v>1645</v>
+        <v>1642</v>
       </c>
       <c r="X265" t="s">
-        <v>49</v>
-      </c>
-      <c r="Y265" t="s">
-        <v>51</v>
+        <v>96</v>
+      </c>
+      <c r="Y265">
+        <v>3</v>
       </c>
       <c r="Z265" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AA265" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AB265" t="s">
-        <v>52</v>
-      </c>
-      <c r="AC265" t="s">
-        <v>53</v>
-      </c>
-      <c r="AD265" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE265" t="s">
-        <v>51</v>
+        <v>53</v>
+      </c>
+      <c r="AC265">
+        <v>3</v>
+      </c>
+      <c r="AD265">
+        <v>3</v>
+      </c>
+      <c r="AE265">
+        <v>3</v>
       </c>
       <c r="AF265" t="s">
         <v>54</v>
@@ -30200,10 +30234,10 @@
     </row>
     <row r="266" spans="1:32">
       <c r="A266" t="s">
-        <v>1633</v>
+        <v>680</v>
       </c>
       <c r="B266" t="s">
-        <v>1634</v>
+        <v>681</v>
       </c>
       <c r="C266" t="s">
         <v>34</v>
@@ -30215,76 +30249,76 @@
         <v>36</v>
       </c>
       <c r="F266" t="s">
-        <v>1646</v>
+        <v>945</v>
       </c>
       <c r="G266" t="s">
-        <v>1647</v>
+        <v>1643</v>
       </c>
       <c r="J266" t="s">
         <v>53</v>
       </c>
       <c r="K266" t="s">
-        <v>239</v>
+        <v>153</v>
       </c>
       <c r="L266" t="s">
-        <v>240</v>
+        <v>154</v>
       </c>
       <c r="M266" t="s">
         <v>42</v>
       </c>
       <c r="N266" t="s">
-        <v>1648</v>
+        <v>892</v>
       </c>
       <c r="O266">
-        <v>120.627419</v>
+        <v>121.466308</v>
       </c>
       <c r="P266">
-        <v>31.311508</v>
+        <v>31.162058</v>
       </c>
       <c r="Q266">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="R266">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="S266" t="s">
         <v>44</v>
       </c>
       <c r="T266" t="s">
-        <v>1216</v>
+        <v>1644</v>
       </c>
       <c r="U266" t="s">
-        <v>1649</v>
+        <v>1645</v>
       </c>
       <c r="V266" t="s">
         <v>47</v>
       </c>
       <c r="W266" t="s">
-        <v>1650</v>
+        <v>1646</v>
       </c>
       <c r="X266" t="s">
         <v>71</v>
       </c>
       <c r="Y266" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Z266" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="AA266" t="s">
         <v>52</v>
       </c>
-      <c r="AB266" t="s">
-        <v>50</v>
+      <c r="AB266">
+        <v>4</v>
       </c>
       <c r="AC266" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="AD266" t="s">
         <v>53</v>
       </c>
-      <c r="AE266" t="s">
-        <v>51</v>
+      <c r="AE266">
+        <v>4</v>
       </c>
       <c r="AF266" t="s">
         <v>54</v>
@@ -30292,10 +30326,10 @@
     </row>
     <row r="267" spans="1:32">
       <c r="A267" t="s">
-        <v>1633</v>
+        <v>680</v>
       </c>
       <c r="B267" t="s">
-        <v>1634</v>
+        <v>681</v>
       </c>
       <c r="C267" t="s">
         <v>34</v>
@@ -30307,67 +30341,67 @@
         <v>36</v>
       </c>
       <c r="F267" t="s">
-        <v>1651</v>
+        <v>1647</v>
       </c>
       <c r="G267" t="s">
-        <v>1652</v>
+        <v>1648</v>
       </c>
       <c r="J267" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="K267" t="s">
-        <v>40</v>
+        <v>370</v>
       </c>
       <c r="L267" t="s">
-        <v>41</v>
+        <v>371</v>
       </c>
       <c r="M267" t="s">
         <v>42</v>
       </c>
       <c r="N267" t="s">
-        <v>1653</v>
+        <v>1649</v>
       </c>
       <c r="O267">
-        <v>120.623497</v>
+        <v>121.466355</v>
       </c>
       <c r="P267">
-        <v>31.304038</v>
+        <v>31.161684</v>
       </c>
       <c r="Q267">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="R267">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="S267" t="s">
         <v>44</v>
       </c>
       <c r="T267" t="s">
-        <v>1654</v>
+        <v>69</v>
       </c>
       <c r="U267" t="s">
-        <v>1655</v>
+        <v>1650</v>
       </c>
       <c r="V267" t="s">
         <v>47</v>
       </c>
       <c r="W267" t="s">
-        <v>1656</v>
+        <v>1651</v>
       </c>
       <c r="X267" t="s">
         <v>49</v>
       </c>
       <c r="Y267" t="s">
-        <v>63</v>
-      </c>
-      <c r="Z267" t="s">
-        <v>51</v>
-      </c>
-      <c r="AA267" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB267" t="s">
-        <v>51</v>
+        <v>50</v>
+      </c>
+      <c r="Z267">
+        <v>4</v>
+      </c>
+      <c r="AA267">
+        <v>3</v>
+      </c>
+      <c r="AB267">
+        <v>3</v>
       </c>
       <c r="AC267" t="s">
         <v>53</v>
@@ -30375,8 +30409,8 @@
       <c r="AD267" t="s">
         <v>53</v>
       </c>
-      <c r="AE267" t="s">
-        <v>63</v>
+      <c r="AE267">
+        <v>4</v>
       </c>
       <c r="AF267" t="s">
         <v>54</v>
@@ -30384,10 +30418,10 @@
     </row>
     <row r="268" spans="1:32">
       <c r="A268" t="s">
-        <v>1633</v>
+        <v>1652</v>
       </c>
       <c r="B268" t="s">
-        <v>1634</v>
+        <v>1653</v>
       </c>
       <c r="C268" t="s">
         <v>34</v>
@@ -30399,34 +30433,37 @@
         <v>36</v>
       </c>
       <c r="F268" t="s">
-        <v>1657</v>
+        <v>1654</v>
       </c>
       <c r="G268" t="s">
-        <v>1658</v>
+        <v>1655</v>
+      </c>
+      <c r="H268" t="s">
+        <v>1656</v>
       </c>
       <c r="J268" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="K268" t="s">
-        <v>480</v>
+        <v>66</v>
       </c>
       <c r="L268" t="s">
-        <v>481</v>
+        <v>67</v>
       </c>
       <c r="M268" t="s">
         <v>42</v>
       </c>
       <c r="N268" t="s">
-        <v>1659</v>
+        <v>1657</v>
       </c>
       <c r="O268">
-        <v>120.63362</v>
+        <v>120.63475</v>
       </c>
       <c r="P268">
-        <v>31.31481</v>
+        <v>31.29909</v>
       </c>
       <c r="Q268">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="R268">
         <v>4.6</v>
@@ -30435,32 +30472,32 @@
         <v>44</v>
       </c>
       <c r="T268" t="s">
-        <v>1660</v>
+        <v>859</v>
       </c>
       <c r="U268" t="s">
-        <v>1661</v>
+        <v>1658</v>
       </c>
       <c r="V268" t="s">
         <v>47</v>
       </c>
       <c r="W268" t="s">
-        <v>1662</v>
+        <v>1659</v>
       </c>
       <c r="X268" t="s">
         <v>71</v>
       </c>
       <c r="Y268" t="s">
+        <v>52</v>
+      </c>
+      <c r="Z268" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA268" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB268" t="s">
         <v>63</v>
       </c>
-      <c r="Z268" t="s">
-        <v>51</v>
-      </c>
-      <c r="AA268" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB268" t="s">
-        <v>52</v>
-      </c>
       <c r="AC268" t="s">
         <v>53</v>
       </c>
@@ -30468,7 +30505,7 @@
         <v>53</v>
       </c>
       <c r="AE268" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="AF268" t="s">
         <v>54</v>
@@ -30476,10 +30513,10 @@
     </row>
     <row r="269" spans="1:32">
       <c r="A269" t="s">
-        <v>1633</v>
+        <v>1652</v>
       </c>
       <c r="B269" t="s">
-        <v>1634</v>
+        <v>1653</v>
       </c>
       <c r="C269" t="s">
         <v>34</v>
@@ -30491,76 +30528,76 @@
         <v>36</v>
       </c>
       <c r="F269" t="s">
-        <v>1663</v>
+        <v>1660</v>
       </c>
       <c r="G269" t="s">
-        <v>1664</v>
+        <v>1661</v>
       </c>
       <c r="J269" t="s">
         <v>53</v>
       </c>
       <c r="K269" t="s">
-        <v>239</v>
+        <v>153</v>
       </c>
       <c r="L269" t="s">
-        <v>240</v>
+        <v>154</v>
       </c>
       <c r="M269" t="s">
         <v>42</v>
       </c>
       <c r="N269" t="s">
-        <v>1665</v>
+        <v>1662</v>
       </c>
       <c r="O269">
-        <v>120.634283</v>
+        <v>120.635604</v>
       </c>
       <c r="P269">
-        <v>31.312167</v>
+        <v>31.306522</v>
       </c>
       <c r="Q269">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="R269">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="S269" t="s">
         <v>44</v>
       </c>
       <c r="T269" t="s">
-        <v>69</v>
+        <v>1052</v>
       </c>
       <c r="U269" t="s">
-        <v>1666</v>
+        <v>1663</v>
       </c>
       <c r="V269" t="s">
         <v>47</v>
       </c>
       <c r="W269" t="s">
-        <v>1667</v>
+        <v>1664</v>
       </c>
       <c r="X269" t="s">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="Y269" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="Z269" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA269" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB269" t="s">
+        <v>52</v>
+      </c>
+      <c r="AC269" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD269" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE269" t="s">
         <v>51</v>
-      </c>
-      <c r="AA269" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB269" t="s">
-        <v>52</v>
-      </c>
-      <c r="AC269" t="s">
-        <v>53</v>
-      </c>
-      <c r="AD269" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE269" t="s">
-        <v>52</v>
       </c>
       <c r="AF269" t="s">
         <v>54</v>
@@ -30568,10 +30605,10 @@
     </row>
     <row r="270" spans="1:32">
       <c r="A270" t="s">
-        <v>1633</v>
+        <v>1652</v>
       </c>
       <c r="B270" t="s">
-        <v>1634</v>
+        <v>1653</v>
       </c>
       <c r="C270" t="s">
         <v>34</v>
@@ -30583,76 +30620,76 @@
         <v>36</v>
       </c>
       <c r="F270" t="s">
-        <v>1668</v>
+        <v>1665</v>
       </c>
       <c r="G270" t="s">
-        <v>1669</v>
+        <v>1666</v>
       </c>
       <c r="J270" t="s">
         <v>53</v>
       </c>
       <c r="K270" t="s">
-        <v>40</v>
+        <v>239</v>
       </c>
       <c r="L270" t="s">
-        <v>41</v>
+        <v>240</v>
       </c>
       <c r="M270" t="s">
         <v>42</v>
       </c>
       <c r="N270" t="s">
-        <v>1670</v>
+        <v>1667</v>
       </c>
       <c r="O270">
-        <v>120.587172</v>
+        <v>120.627419</v>
       </c>
       <c r="P270">
-        <v>31.314389</v>
+        <v>31.311508</v>
       </c>
       <c r="Q270">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="R270">
-        <v>4.7</v>
+        <v>4.5</v>
       </c>
       <c r="S270" t="s">
         <v>44</v>
       </c>
       <c r="T270" t="s">
-        <v>1671</v>
+        <v>1216</v>
       </c>
       <c r="U270" t="s">
-        <v>1672</v>
+        <v>1668</v>
       </c>
       <c r="V270" t="s">
         <v>47</v>
       </c>
       <c r="W270" t="s">
-        <v>1673</v>
+        <v>1669</v>
       </c>
       <c r="X270" t="s">
-        <v>49</v>
+        <v>71</v>
       </c>
       <c r="Y270" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z270" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA270" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB270" t="s">
         <v>50</v>
       </c>
-      <c r="Z270" t="s">
-        <v>52</v>
-      </c>
-      <c r="AA270" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB270" t="s">
+      <c r="AC270" t="s">
         <v>51</v>
       </c>
-      <c r="AC270" t="s">
-        <v>53</v>
-      </c>
       <c r="AD270" t="s">
         <v>53</v>
       </c>
       <c r="AE270" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AF270" t="s">
         <v>54</v>
@@ -30660,10 +30697,10 @@
     </row>
     <row r="271" spans="1:32">
       <c r="A271" t="s">
-        <v>1633</v>
+        <v>1652</v>
       </c>
       <c r="B271" t="s">
-        <v>1634</v>
+        <v>1653</v>
       </c>
       <c r="C271" t="s">
         <v>34</v>
@@ -30675,73 +30712,73 @@
         <v>36</v>
       </c>
       <c r="F271" t="s">
-        <v>1674</v>
+        <v>1670</v>
       </c>
       <c r="G271" t="s">
-        <v>1675</v>
+        <v>1671</v>
       </c>
       <c r="J271" t="s">
         <v>53</v>
       </c>
       <c r="K271" t="s">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="L271" t="s">
-        <v>91</v>
+        <v>41</v>
       </c>
       <c r="M271" t="s">
         <v>42</v>
       </c>
       <c r="N271" t="s">
-        <v>1676</v>
+        <v>1672</v>
       </c>
       <c r="O271">
-        <v>120.622713</v>
+        <v>120.623497</v>
       </c>
       <c r="P271">
-        <v>31.30227</v>
+        <v>31.304038</v>
       </c>
       <c r="Q271">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="R271">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="S271" t="s">
         <v>44</v>
       </c>
       <c r="T271" t="s">
-        <v>1677</v>
+        <v>1673</v>
       </c>
       <c r="U271" t="s">
-        <v>1678</v>
+        <v>1674</v>
       </c>
       <c r="V271" t="s">
         <v>47</v>
       </c>
       <c r="W271" t="s">
-        <v>1679</v>
+        <v>1675</v>
       </c>
       <c r="X271" t="s">
-        <v>96</v>
+        <v>49</v>
       </c>
       <c r="Y271" t="s">
         <v>63</v>
       </c>
       <c r="Z271" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="AA271" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AB271" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="AC271" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AD271" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AE271" t="s">
         <v>63</v>
@@ -30752,10 +30789,10 @@
     </row>
     <row r="272" spans="1:32">
       <c r="A272" t="s">
-        <v>1633</v>
+        <v>1652</v>
       </c>
       <c r="B272" t="s">
-        <v>1634</v>
+        <v>1653</v>
       </c>
       <c r="C272" t="s">
         <v>34</v>
@@ -30767,73 +30804,73 @@
         <v>36</v>
       </c>
       <c r="F272" t="s">
-        <v>1680</v>
+        <v>1676</v>
       </c>
       <c r="G272" t="s">
-        <v>1681</v>
+        <v>1677</v>
       </c>
       <c r="J272" t="s">
         <v>39</v>
       </c>
       <c r="K272" t="s">
-        <v>301</v>
+        <v>480</v>
       </c>
       <c r="L272" t="s">
-        <v>302</v>
+        <v>481</v>
       </c>
       <c r="M272" t="s">
         <v>42</v>
       </c>
       <c r="N272" t="s">
-        <v>1682</v>
+        <v>1678</v>
       </c>
       <c r="O272">
-        <v>120.627239</v>
+        <v>120.63362</v>
       </c>
       <c r="P272">
-        <v>31.301281</v>
+        <v>31.31481</v>
       </c>
       <c r="Q272">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="R272">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="S272" t="s">
         <v>44</v>
       </c>
       <c r="T272" t="s">
-        <v>1253</v>
+        <v>1679</v>
       </c>
       <c r="U272" t="s">
-        <v>1683</v>
+        <v>1680</v>
       </c>
       <c r="V272" t="s">
         <v>47</v>
       </c>
       <c r="W272" t="s">
-        <v>1684</v>
+        <v>1681</v>
       </c>
       <c r="X272" t="s">
-        <v>96</v>
+        <v>71</v>
       </c>
       <c r="Y272" t="s">
         <v>63</v>
       </c>
       <c r="Z272" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="AA272" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AB272" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AC272" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AD272" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AE272" t="s">
         <v>63</v>
@@ -30844,10 +30881,10 @@
     </row>
     <row r="273" spans="1:32">
       <c r="A273" t="s">
-        <v>1633</v>
+        <v>1652</v>
       </c>
       <c r="B273" t="s">
-        <v>1634</v>
+        <v>1653</v>
       </c>
       <c r="C273" t="s">
         <v>34</v>
@@ -30859,67 +30896,67 @@
         <v>36</v>
       </c>
       <c r="F273" t="s">
-        <v>1617</v>
+        <v>1682</v>
       </c>
       <c r="G273" t="s">
-        <v>1685</v>
+        <v>1683</v>
       </c>
       <c r="J273" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="K273" t="s">
-        <v>40</v>
+        <v>239</v>
       </c>
       <c r="L273" t="s">
-        <v>41</v>
+        <v>240</v>
       </c>
       <c r="M273" t="s">
         <v>42</v>
       </c>
       <c r="N273" t="s">
-        <v>1686</v>
+        <v>1684</v>
       </c>
       <c r="O273">
-        <v>120.765532</v>
+        <v>120.634283</v>
       </c>
       <c r="P273">
-        <v>31.305686</v>
+        <v>31.312167</v>
       </c>
       <c r="Q273">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="R273">
-        <v>4.4</v>
+        <v>4.7</v>
       </c>
       <c r="S273" t="s">
         <v>44</v>
       </c>
       <c r="T273" t="s">
-        <v>1687</v>
+        <v>69</v>
       </c>
       <c r="U273" t="s">
-        <v>1688</v>
+        <v>1685</v>
       </c>
       <c r="V273" t="s">
         <v>47</v>
       </c>
       <c r="W273" t="s">
-        <v>1689</v>
+        <v>1686</v>
       </c>
       <c r="X273" t="s">
-        <v>49</v>
+        <v>71</v>
       </c>
       <c r="Y273" t="s">
+        <v>52</v>
+      </c>
+      <c r="Z273" t="s">
         <v>51</v>
       </c>
-      <c r="Z273" t="s">
-        <v>52</v>
-      </c>
       <c r="AA273" t="s">
         <v>52</v>
       </c>
       <c r="AB273" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="AC273" t="s">
         <v>53</v>
@@ -30928,7 +30965,7 @@
         <v>53</v>
       </c>
       <c r="AE273" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AF273" t="s">
         <v>54</v>
@@ -30936,10 +30973,10 @@
     </row>
     <row r="274" spans="1:32">
       <c r="A274" t="s">
-        <v>1633</v>
+        <v>1652</v>
       </c>
       <c r="B274" t="s">
-        <v>1634</v>
+        <v>1653</v>
       </c>
       <c r="C274" t="s">
         <v>34</v>
@@ -30951,76 +30988,76 @@
         <v>36</v>
       </c>
       <c r="F274" t="s">
-        <v>1690</v>
+        <v>1687</v>
       </c>
       <c r="G274" t="s">
-        <v>1691</v>
+        <v>1688</v>
       </c>
       <c r="J274" t="s">
         <v>53</v>
       </c>
       <c r="K274" t="s">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="L274" t="s">
-        <v>91</v>
+        <v>41</v>
       </c>
       <c r="M274" t="s">
         <v>42</v>
       </c>
       <c r="N274" t="s">
-        <v>1692</v>
+        <v>1689</v>
       </c>
       <c r="O274">
-        <v>120.598498</v>
+        <v>120.587172</v>
       </c>
       <c r="P274">
-        <v>31.320662</v>
+        <v>31.314389</v>
       </c>
       <c r="Q274">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R274">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="S274" t="s">
         <v>44</v>
       </c>
       <c r="T274" t="s">
-        <v>1693</v>
+        <v>1690</v>
       </c>
       <c r="U274" t="s">
-        <v>1694</v>
+        <v>1691</v>
       </c>
       <c r="V274" t="s">
         <v>47</v>
       </c>
       <c r="W274" t="s">
-        <v>1695</v>
+        <v>1692</v>
       </c>
       <c r="X274" t="s">
-        <v>96</v>
+        <v>49</v>
       </c>
       <c r="Y274" t="s">
+        <v>50</v>
+      </c>
+      <c r="Z274" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA274" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB274" t="s">
         <v>51</v>
       </c>
-      <c r="Z274" t="s">
-        <v>53</v>
-      </c>
-      <c r="AA274" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB274" t="s">
-        <v>53</v>
-      </c>
       <c r="AC274" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="AD274" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AE274" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AF274" t="s">
         <v>54</v>
@@ -31028,10 +31065,10 @@
     </row>
     <row r="275" spans="1:32">
       <c r="A275" t="s">
-        <v>1696</v>
+        <v>1652</v>
       </c>
       <c r="B275" t="s">
-        <v>1697</v>
+        <v>1653</v>
       </c>
       <c r="C275" t="s">
         <v>34</v>
@@ -31043,58 +31080,58 @@
         <v>36</v>
       </c>
       <c r="F275" t="s">
-        <v>1085</v>
+        <v>1693</v>
       </c>
       <c r="G275" t="s">
-        <v>1698</v>
+        <v>1694</v>
       </c>
       <c r="J275" t="s">
         <v>53</v>
       </c>
       <c r="K275" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="L275" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="M275" t="s">
         <v>42</v>
       </c>
       <c r="N275" t="s">
-        <v>1699</v>
+        <v>1695</v>
       </c>
       <c r="O275">
-        <v>118.080176</v>
+        <v>120.622713</v>
       </c>
       <c r="P275">
-        <v>24.453843</v>
+        <v>31.30227</v>
       </c>
       <c r="Q275">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="R275">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="S275" t="s">
         <v>44</v>
       </c>
       <c r="T275" t="s">
-        <v>869</v>
+        <v>1696</v>
       </c>
       <c r="U275" t="s">
-        <v>1700</v>
+        <v>1697</v>
       </c>
       <c r="V275" t="s">
         <v>47</v>
       </c>
       <c r="W275" t="s">
-        <v>1701</v>
+        <v>1698</v>
       </c>
       <c r="X275" t="s">
         <v>96</v>
       </c>
       <c r="Y275" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="Z275" t="s">
         <v>53</v>
@@ -31106,13 +31143,13 @@
         <v>53</v>
       </c>
       <c r="AC275" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AD275" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AE275" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="AF275" t="s">
         <v>54</v>
@@ -31120,10 +31157,10 @@
     </row>
     <row r="276" spans="1:32">
       <c r="A276" t="s">
-        <v>1696</v>
+        <v>1652</v>
       </c>
       <c r="B276" t="s">
-        <v>1697</v>
+        <v>1653</v>
       </c>
       <c r="C276" t="s">
         <v>34</v>
@@ -31135,76 +31172,76 @@
         <v>36</v>
       </c>
       <c r="F276" t="s">
-        <v>1702</v>
+        <v>1699</v>
       </c>
       <c r="G276" t="s">
-        <v>1703</v>
+        <v>1700</v>
       </c>
       <c r="J276" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="K276" t="s">
-        <v>370</v>
+        <v>301</v>
       </c>
       <c r="L276" t="s">
-        <v>371</v>
+        <v>302</v>
       </c>
       <c r="M276" t="s">
         <v>42</v>
       </c>
       <c r="N276" t="s">
-        <v>1704</v>
+        <v>1701</v>
       </c>
       <c r="O276">
-        <v>118.083631</v>
+        <v>120.627239</v>
       </c>
       <c r="P276">
-        <v>24.451722</v>
+        <v>31.301281</v>
       </c>
       <c r="Q276">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="R276">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="S276" t="s">
         <v>44</v>
       </c>
       <c r="T276" t="s">
-        <v>1705</v>
+        <v>1253</v>
       </c>
       <c r="U276" t="s">
-        <v>1706</v>
+        <v>1702</v>
       </c>
       <c r="V276" t="s">
         <v>47</v>
       </c>
       <c r="W276" t="s">
-        <v>1707</v>
+        <v>1703</v>
       </c>
       <c r="X276" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="Y276" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="Z276" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AA276" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AB276" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="AC276" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AD276" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AE276" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="AF276" t="s">
         <v>54</v>
@@ -31212,10 +31249,10 @@
     </row>
     <row r="277" spans="1:32">
       <c r="A277" t="s">
-        <v>1696</v>
+        <v>1652</v>
       </c>
       <c r="B277" t="s">
-        <v>1697</v>
+        <v>1653</v>
       </c>
       <c r="C277" t="s">
         <v>34</v>
@@ -31227,13 +31264,13 @@
         <v>36</v>
       </c>
       <c r="F277" t="s">
-        <v>1708</v>
+        <v>1617</v>
       </c>
       <c r="G277" t="s">
-        <v>1709</v>
+        <v>1704</v>
       </c>
       <c r="J277" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="K277" t="s">
         <v>40</v>
@@ -31245,49 +31282,49 @@
         <v>42</v>
       </c>
       <c r="N277" t="s">
-        <v>1710</v>
+        <v>1705</v>
       </c>
       <c r="O277">
-        <v>118.078485</v>
+        <v>120.765532</v>
       </c>
       <c r="P277">
-        <v>24.453691</v>
+        <v>31.305686</v>
       </c>
       <c r="Q277">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="R277">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="S277" t="s">
         <v>44</v>
       </c>
       <c r="T277" t="s">
-        <v>1711</v>
+        <v>1706</v>
       </c>
       <c r="U277" t="s">
-        <v>1712</v>
+        <v>1707</v>
       </c>
       <c r="V277" t="s">
         <v>47</v>
       </c>
       <c r="W277" t="s">
-        <v>1713</v>
+        <v>1708</v>
       </c>
       <c r="X277" t="s">
         <v>49</v>
       </c>
       <c r="Y277" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="Z277" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AA277" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AB277" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="AC277" t="s">
         <v>53</v>
@@ -31296,7 +31333,7 @@
         <v>53</v>
       </c>
       <c r="AE277" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="AF277" t="s">
         <v>54</v>
@@ -31304,10 +31341,10 @@
     </row>
     <row r="278" spans="1:32">
       <c r="A278" t="s">
-        <v>1696</v>
+        <v>1652</v>
       </c>
       <c r="B278" t="s">
-        <v>1697</v>
+        <v>1653</v>
       </c>
       <c r="C278" t="s">
         <v>34</v>
@@ -31319,76 +31356,76 @@
         <v>36</v>
       </c>
       <c r="F278" t="s">
-        <v>1714</v>
+        <v>1709</v>
       </c>
       <c r="G278" t="s">
-        <v>1715</v>
+        <v>1710</v>
       </c>
       <c r="J278" t="s">
         <v>53</v>
       </c>
       <c r="K278" t="s">
-        <v>193</v>
+        <v>90</v>
       </c>
       <c r="L278" t="s">
-        <v>194</v>
+        <v>91</v>
       </c>
       <c r="M278" t="s">
         <v>42</v>
       </c>
       <c r="N278" t="s">
-        <v>1716</v>
+        <v>1711</v>
       </c>
       <c r="O278">
-        <v>118.088965</v>
+        <v>120.598498</v>
       </c>
       <c r="P278">
-        <v>24.438235</v>
+        <v>31.320662</v>
       </c>
       <c r="Q278">
-        <v>62</v>
+        <v>15</v>
       </c>
       <c r="R278">
-        <v>4.2</v>
+        <v>4.6</v>
       </c>
       <c r="S278" t="s">
         <v>44</v>
       </c>
       <c r="T278" t="s">
-        <v>156</v>
+        <v>1712</v>
       </c>
       <c r="U278" t="s">
-        <v>1717</v>
+        <v>1713</v>
       </c>
       <c r="V278" t="s">
         <v>47</v>
       </c>
       <c r="W278" t="s">
-        <v>1718</v>
+        <v>1714</v>
       </c>
       <c r="X278" t="s">
-        <v>49</v>
+        <v>96</v>
       </c>
       <c r="Y278" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="Z278" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AA278" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AB278" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="AC278" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="AD278" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AE278" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="AF278" t="s">
         <v>54</v>
@@ -31396,10 +31433,10 @@
     </row>
     <row r="279" spans="1:32">
       <c r="A279" t="s">
-        <v>1719</v>
+        <v>1715</v>
       </c>
       <c r="B279" t="s">
-        <v>1720</v>
+        <v>1716</v>
       </c>
       <c r="C279" t="s">
         <v>34</v>
@@ -31411,67 +31448,67 @@
         <v>36</v>
       </c>
       <c r="F279" t="s">
-        <v>1721</v>
+        <v>1085</v>
       </c>
       <c r="G279" t="s">
-        <v>1722</v>
+        <v>1717</v>
       </c>
       <c r="J279" t="s">
         <v>53</v>
       </c>
       <c r="K279" t="s">
-        <v>1158</v>
+        <v>66</v>
       </c>
       <c r="L279" t="s">
-        <v>1159</v>
+        <v>67</v>
       </c>
       <c r="M279" t="s">
         <v>42</v>
       </c>
       <c r="N279" t="s">
-        <v>1723</v>
-      </c>
-      <c r="O279" t="s">
-        <v>1724</v>
-      </c>
-      <c r="P279" t="s">
-        <v>1725</v>
+        <v>1718</v>
+      </c>
+      <c r="O279">
+        <v>118.080176</v>
+      </c>
+      <c r="P279">
+        <v>24.453843</v>
       </c>
       <c r="Q279">
-        <v>71</v>
+        <v>17</v>
       </c>
       <c r="R279">
-        <v>4.6</v>
+        <v>4.5</v>
       </c>
       <c r="S279" t="s">
         <v>44</v>
       </c>
       <c r="T279" t="s">
-        <v>1726</v>
+        <v>869</v>
       </c>
       <c r="U279" t="s">
-        <v>1727</v>
+        <v>1719</v>
       </c>
       <c r="V279" t="s">
         <v>47</v>
       </c>
       <c r="W279" t="s">
-        <v>1728</v>
+        <v>1720</v>
       </c>
       <c r="X279" t="s">
-        <v>49</v>
-      </c>
-      <c r="Y279">
-        <v>3</v>
-      </c>
-      <c r="Z279">
-        <v>4</v>
+        <v>96</v>
+      </c>
+      <c r="Y279" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z279" t="s">
+        <v>53</v>
       </c>
       <c r="AA279" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB279">
-        <v>2</v>
+        <v>53</v>
+      </c>
+      <c r="AB279" t="s">
+        <v>53</v>
       </c>
       <c r="AC279" t="s">
         <v>53</v>
@@ -31479,8 +31516,8 @@
       <c r="AD279" t="s">
         <v>53</v>
       </c>
-      <c r="AE279">
-        <v>3</v>
+      <c r="AE279" t="s">
+        <v>53</v>
       </c>
       <c r="AF279" t="s">
         <v>54</v>
@@ -31488,10 +31525,10 @@
     </row>
     <row r="280" spans="1:32">
       <c r="A280" t="s">
-        <v>1719</v>
+        <v>1715</v>
       </c>
       <c r="B280" t="s">
-        <v>1720</v>
+        <v>1716</v>
       </c>
       <c r="C280" t="s">
         <v>34</v>
@@ -31506,73 +31543,73 @@
         <v>1721</v>
       </c>
       <c r="G280" t="s">
-        <v>1729</v>
+        <v>1722</v>
       </c>
       <c r="J280" t="s">
         <v>53</v>
       </c>
       <c r="K280" t="s">
-        <v>1158</v>
+        <v>370</v>
       </c>
       <c r="L280" t="s">
-        <v>1159</v>
+        <v>371</v>
       </c>
       <c r="M280" t="s">
         <v>42</v>
       </c>
       <c r="N280" t="s">
-        <v>1730</v>
-      </c>
-      <c r="O280" t="s">
-        <v>1731</v>
-      </c>
-      <c r="P280" t="s">
-        <v>1732</v>
+        <v>1723</v>
+      </c>
+      <c r="O280">
+        <v>118.083631</v>
+      </c>
+      <c r="P280">
+        <v>24.451722</v>
       </c>
       <c r="Q280">
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="R280">
-        <v>4.6</v>
+        <v>4.2</v>
       </c>
       <c r="S280" t="s">
         <v>44</v>
       </c>
       <c r="T280" t="s">
-        <v>1733</v>
+        <v>1724</v>
       </c>
       <c r="U280" t="s">
-        <v>1734</v>
+        <v>1725</v>
       </c>
       <c r="V280" t="s">
         <v>47</v>
       </c>
       <c r="W280" t="s">
-        <v>1735</v>
+        <v>1726</v>
       </c>
       <c r="X280" t="s">
-        <v>49</v>
-      </c>
-      <c r="Y280">
-        <v>3</v>
-      </c>
-      <c r="Z280">
-        <v>4</v>
+        <v>71</v>
+      </c>
+      <c r="Y280" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z280" t="s">
+        <v>52</v>
       </c>
       <c r="AA280" t="s">
         <v>52</v>
       </c>
-      <c r="AB280">
-        <v>2</v>
+      <c r="AB280" t="s">
+        <v>50</v>
       </c>
       <c r="AC280" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="AD280" t="s">
         <v>53</v>
       </c>
-      <c r="AE280">
-        <v>3</v>
+      <c r="AE280" t="s">
+        <v>51</v>
       </c>
       <c r="AF280" t="s">
         <v>54</v>
@@ -31580,10 +31617,10 @@
     </row>
     <row r="281" spans="1:32">
       <c r="A281" t="s">
-        <v>1719</v>
+        <v>1715</v>
       </c>
       <c r="B281" t="s">
-        <v>1720</v>
+        <v>1716</v>
       </c>
       <c r="C281" t="s">
         <v>34</v>
@@ -31595,76 +31632,76 @@
         <v>36</v>
       </c>
       <c r="F281" t="s">
-        <v>1736</v>
+        <v>1727</v>
       </c>
       <c r="G281" t="s">
-        <v>1737</v>
+        <v>1728</v>
       </c>
       <c r="J281" t="s">
         <v>53</v>
       </c>
       <c r="K281" t="s">
-        <v>239</v>
+        <v>40</v>
       </c>
       <c r="L281" t="s">
-        <v>240</v>
+        <v>41</v>
       </c>
       <c r="M281" t="s">
         <v>42</v>
       </c>
       <c r="N281" t="s">
-        <v>1738</v>
-      </c>
-      <c r="O281" t="s">
-        <v>1739</v>
-      </c>
-      <c r="P281" t="s">
-        <v>1740</v>
+        <v>1729</v>
+      </c>
+      <c r="O281">
+        <v>118.078485</v>
+      </c>
+      <c r="P281">
+        <v>24.453691</v>
       </c>
       <c r="Q281">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="R281">
-        <v>4.6</v>
+        <v>4.5</v>
       </c>
       <c r="S281" t="s">
         <v>44</v>
       </c>
       <c r="T281" t="s">
-        <v>726</v>
+        <v>1730</v>
       </c>
       <c r="U281" t="s">
-        <v>1741</v>
+        <v>1731</v>
       </c>
       <c r="V281" t="s">
         <v>47</v>
       </c>
       <c r="W281" t="s">
-        <v>1742</v>
+        <v>1732</v>
       </c>
       <c r="X281" t="s">
-        <v>71</v>
-      </c>
-      <c r="Y281">
-        <v>4</v>
+        <v>49</v>
+      </c>
+      <c r="Y281" t="s">
+        <v>53</v>
       </c>
       <c r="Z281" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AA281" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB281">
-        <v>3</v>
-      </c>
-      <c r="AC281">
-        <v>3</v>
+        <v>53</v>
+      </c>
+      <c r="AB281" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC281" t="s">
+        <v>53</v>
       </c>
       <c r="AD281" t="s">
         <v>53</v>
       </c>
-      <c r="AE281">
-        <v>3</v>
+      <c r="AE281" t="s">
+        <v>53</v>
       </c>
       <c r="AF281" t="s">
         <v>54</v>
@@ -31672,10 +31709,10 @@
     </row>
     <row r="282" spans="1:32">
       <c r="A282" t="s">
-        <v>1719</v>
+        <v>1715</v>
       </c>
       <c r="B282" t="s">
-        <v>1720</v>
+        <v>1716</v>
       </c>
       <c r="C282" t="s">
         <v>34</v>
@@ -31687,52 +31724,52 @@
         <v>36</v>
       </c>
       <c r="F282" t="s">
-        <v>1743</v>
+        <v>1733</v>
       </c>
       <c r="G282" t="s">
-        <v>1744</v>
+        <v>1734</v>
       </c>
       <c r="J282" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="K282" t="s">
-        <v>82</v>
+        <v>193</v>
       </c>
       <c r="L282" t="s">
-        <v>83</v>
+        <v>194</v>
       </c>
       <c r="M282" t="s">
         <v>42</v>
       </c>
       <c r="N282" t="s">
-        <v>1745</v>
-      </c>
-      <c r="O282" t="s">
-        <v>1746</v>
-      </c>
-      <c r="P282" t="s">
-        <v>1747</v>
+        <v>1735</v>
+      </c>
+      <c r="O282">
+        <v>118.088965</v>
+      </c>
+      <c r="P282">
+        <v>24.438235</v>
       </c>
       <c r="Q282">
-        <v>121</v>
+        <v>62</v>
       </c>
       <c r="R282">
-        <v>4.7</v>
+        <v>4.2</v>
       </c>
       <c r="S282" t="s">
         <v>44</v>
       </c>
       <c r="T282" t="s">
-        <v>1748</v>
+        <v>156</v>
       </c>
       <c r="U282" t="s">
-        <v>1749</v>
+        <v>1736</v>
       </c>
       <c r="V282" t="s">
         <v>47</v>
       </c>
       <c r="W282" t="s">
-        <v>1750</v>
+        <v>1737</v>
       </c>
       <c r="X282" t="s">
         <v>49</v>
@@ -31740,14 +31777,14 @@
       <c r="Y282" t="s">
         <v>63</v>
       </c>
-      <c r="Z282">
-        <v>4</v>
+      <c r="Z282" t="s">
+        <v>52</v>
       </c>
       <c r="AA282" t="s">
         <v>52</v>
       </c>
-      <c r="AB282">
-        <v>3</v>
+      <c r="AB282" t="s">
+        <v>50</v>
       </c>
       <c r="AC282" t="s">
         <v>53</v>
@@ -31764,10 +31801,10 @@
     </row>
     <row r="283" spans="1:32">
       <c r="A283" t="s">
-        <v>1719</v>
+        <v>1738</v>
       </c>
       <c r="B283" t="s">
-        <v>1720</v>
+        <v>1739</v>
       </c>
       <c r="C283" t="s">
         <v>34</v>
@@ -31779,67 +31816,70 @@
         <v>36</v>
       </c>
       <c r="F283" t="s">
-        <v>64</v>
+        <v>1740</v>
       </c>
       <c r="G283" t="s">
-        <v>1751</v>
+        <v>1741</v>
       </c>
       <c r="J283" t="s">
         <v>53</v>
       </c>
       <c r="K283" t="s">
-        <v>66</v>
+        <v>1158</v>
       </c>
       <c r="L283" t="s">
-        <v>67</v>
+        <v>1159</v>
       </c>
       <c r="M283" t="s">
         <v>42</v>
       </c>
       <c r="N283" t="s">
-        <v>1752</v>
+        <v>1742</v>
       </c>
       <c r="O283" t="s">
-        <v>1753</v>
+        <v>1743</v>
       </c>
       <c r="P283" t="s">
-        <v>1754</v>
+        <v>1744</v>
       </c>
       <c r="Q283">
-        <v>18</v>
+        <v>71</v>
       </c>
       <c r="R283">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="S283" t="s">
         <v>44</v>
       </c>
       <c r="T283" t="s">
-        <v>869</v>
+        <v>1745</v>
+      </c>
+      <c r="U283" t="s">
+        <v>1746</v>
       </c>
       <c r="V283" t="s">
         <v>47</v>
       </c>
       <c r="W283" t="s">
-        <v>1755</v>
+        <v>1747</v>
       </c>
       <c r="X283" t="s">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="Y283">
         <v>3</v>
       </c>
-      <c r="Z283" t="s">
-        <v>52</v>
+      <c r="Z283">
+        <v>4</v>
       </c>
       <c r="AA283" t="s">
         <v>52</v>
       </c>
       <c r="AB283">
-        <v>3</v>
-      </c>
-      <c r="AC283">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="AC283" t="s">
+        <v>53</v>
       </c>
       <c r="AD283" t="s">
         <v>53</v>
@@ -31853,10 +31893,10 @@
     </row>
     <row r="284" spans="1:32">
       <c r="A284" t="s">
-        <v>1719</v>
+        <v>1738</v>
       </c>
       <c r="B284" t="s">
-        <v>1720</v>
+        <v>1739</v>
       </c>
       <c r="C284" t="s">
         <v>34</v>
@@ -31868,34 +31908,34 @@
         <v>36</v>
       </c>
       <c r="F284" t="s">
-        <v>1756</v>
+        <v>1740</v>
       </c>
       <c r="G284" t="s">
-        <v>1757</v>
+        <v>1748</v>
       </c>
       <c r="J284" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="K284" t="s">
-        <v>239</v>
+        <v>1158</v>
       </c>
       <c r="L284" t="s">
-        <v>240</v>
+        <v>1159</v>
       </c>
       <c r="M284" t="s">
         <v>42</v>
       </c>
       <c r="N284" t="s">
-        <v>1758</v>
+        <v>1749</v>
       </c>
       <c r="O284" t="s">
-        <v>1759</v>
+        <v>1750</v>
       </c>
       <c r="P284" t="s">
-        <v>1760</v>
+        <v>1751</v>
       </c>
       <c r="Q284">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="R284">
         <v>4.6</v>
@@ -31904,40 +31944,40 @@
         <v>44</v>
       </c>
       <c r="T284" t="s">
-        <v>1761</v>
+        <v>1752</v>
       </c>
       <c r="U284" t="s">
-        <v>1762</v>
+        <v>1753</v>
       </c>
       <c r="V284" t="s">
         <v>47</v>
       </c>
       <c r="W284" t="s">
-        <v>1763</v>
+        <v>1754</v>
       </c>
       <c r="X284" t="s">
         <v>49</v>
       </c>
       <c r="Y284">
+        <v>3</v>
+      </c>
+      <c r="Z284">
         <v>4</v>
       </c>
-      <c r="Z284">
+      <c r="AA284" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB284">
         <v>2</v>
       </c>
-      <c r="AA284" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB284">
+      <c r="AC284" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD284" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE284">
         <v>3</v>
-      </c>
-      <c r="AC284" t="s">
-        <v>53</v>
-      </c>
-      <c r="AD284" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE284">
-        <v>4</v>
       </c>
       <c r="AF284" t="s">
         <v>54</v>
@@ -31945,10 +31985,10 @@
     </row>
     <row r="285" spans="1:32">
       <c r="A285" t="s">
-        <v>1719</v>
+        <v>1738</v>
       </c>
       <c r="B285" t="s">
-        <v>1720</v>
+        <v>1739</v>
       </c>
       <c r="C285" t="s">
         <v>34</v>
@@ -31960,70 +32000,70 @@
         <v>36</v>
       </c>
       <c r="F285" t="s">
-        <v>1764</v>
+        <v>1755</v>
       </c>
       <c r="G285" t="s">
-        <v>1765</v>
+        <v>1756</v>
       </c>
       <c r="J285" t="s">
         <v>53</v>
       </c>
       <c r="K285" t="s">
-        <v>351</v>
+        <v>239</v>
       </c>
       <c r="L285" t="s">
-        <v>352</v>
+        <v>240</v>
       </c>
       <c r="M285" t="s">
         <v>42</v>
       </c>
       <c r="N285" t="s">
-        <v>1766</v>
+        <v>1757</v>
       </c>
       <c r="O285" t="s">
-        <v>1767</v>
+        <v>1758</v>
       </c>
       <c r="P285" t="s">
-        <v>1768</v>
+        <v>1759</v>
       </c>
       <c r="Q285">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="R285">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="S285" t="s">
         <v>44</v>
       </c>
       <c r="T285" t="s">
-        <v>985</v>
+        <v>726</v>
       </c>
       <c r="U285" t="s">
-        <v>1769</v>
+        <v>1760</v>
       </c>
       <c r="V285" t="s">
         <v>47</v>
       </c>
       <c r="W285" t="s">
-        <v>1770</v>
+        <v>1761</v>
       </c>
       <c r="X285" t="s">
-        <v>49</v>
+        <v>71</v>
       </c>
       <c r="Y285">
+        <v>4</v>
+      </c>
+      <c r="Z285" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA285" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB285">
         <v>3</v>
       </c>
-      <c r="Z285">
-        <v>2</v>
-      </c>
-      <c r="AA285">
-        <v>2</v>
-      </c>
-      <c r="AB285">
-        <v>4</v>
-      </c>
-      <c r="AC285" t="s">
-        <v>53</v>
+      <c r="AC285">
+        <v>3</v>
       </c>
       <c r="AD285" t="s">
         <v>53</v>
@@ -32037,10 +32077,10 @@
     </row>
     <row r="286" spans="1:32">
       <c r="A286" t="s">
-        <v>1719</v>
+        <v>1738</v>
       </c>
       <c r="B286" t="s">
-        <v>1720</v>
+        <v>1739</v>
       </c>
       <c r="C286" t="s">
         <v>34</v>
@@ -32052,87 +32092,87 @@
         <v>36</v>
       </c>
       <c r="F286" t="s">
-        <v>1771</v>
+        <v>1762</v>
       </c>
       <c r="G286" t="s">
-        <v>1772</v>
+        <v>1763</v>
       </c>
       <c r="J286" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="K286" t="s">
-        <v>193</v>
+        <v>82</v>
       </c>
       <c r="L286" t="s">
-        <v>194</v>
+        <v>83</v>
       </c>
       <c r="M286" t="s">
         <v>42</v>
       </c>
       <c r="N286" t="s">
-        <v>1773</v>
+        <v>1764</v>
       </c>
       <c r="O286" t="s">
-        <v>1774</v>
+        <v>1765</v>
       </c>
       <c r="P286" t="s">
-        <v>1775</v>
+        <v>1766</v>
       </c>
       <c r="Q286">
-        <v>33</v>
+        <v>121</v>
       </c>
       <c r="R286">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="S286" t="s">
         <v>44</v>
       </c>
       <c r="T286" t="s">
-        <v>1776</v>
+        <v>1767</v>
       </c>
       <c r="U286" t="s">
-        <v>1777</v>
+        <v>1768</v>
       </c>
       <c r="V286" t="s">
         <v>47</v>
       </c>
       <c r="W286" t="s">
-        <v>1778</v>
+        <v>1769</v>
       </c>
       <c r="X286" t="s">
         <v>49</v>
       </c>
-      <c r="Y286">
+      <c r="Y286" t="s">
+        <v>63</v>
+      </c>
+      <c r="Z286">
+        <v>4</v>
+      </c>
+      <c r="AA286" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB286">
         <v>3</v>
       </c>
-      <c r="Z286" t="s">
-        <v>52</v>
-      </c>
-      <c r="AA286" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB286" t="s">
-        <v>50</v>
-      </c>
       <c r="AC286" t="s">
         <v>53</v>
       </c>
       <c r="AD286" t="s">
         <v>53</v>
       </c>
-      <c r="AE286">
-        <v>3</v>
+      <c r="AE286" t="s">
+        <v>63</v>
       </c>
       <c r="AF286" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="287" customFormat="1" spans="1:32">
+    <row r="287" spans="1:32">
       <c r="A287" t="s">
-        <v>1719</v>
+        <v>1738</v>
       </c>
       <c r="B287" t="s">
-        <v>1720</v>
+        <v>1739</v>
       </c>
       <c r="C287" t="s">
         <v>34</v>
@@ -32144,10 +32184,10 @@
         <v>36</v>
       </c>
       <c r="F287" t="s">
-        <v>1779</v>
+        <v>64</v>
       </c>
       <c r="G287" t="s">
-        <v>1780</v>
+        <v>1770</v>
       </c>
       <c r="J287" t="s">
         <v>53</v>
@@ -32162,17 +32202,32 @@
         <v>42</v>
       </c>
       <c r="N287" t="s">
-        <v>436</v>
-      </c>
-      <c r="O287"/>
-      <c r="P287"/>
-      <c r="Q287"/>
-      <c r="R287"/>
-      <c r="S287"/>
-      <c r="T287"/>
-      <c r="U287"/>
-      <c r="V287"/>
-      <c r="W287"/>
+        <v>1771</v>
+      </c>
+      <c r="O287" t="s">
+        <v>1772</v>
+      </c>
+      <c r="P287" t="s">
+        <v>1773</v>
+      </c>
+      <c r="Q287">
+        <v>18</v>
+      </c>
+      <c r="R287">
+        <v>4.7</v>
+      </c>
+      <c r="S287" t="s">
+        <v>44</v>
+      </c>
+      <c r="T287" t="s">
+        <v>869</v>
+      </c>
+      <c r="V287" t="s">
+        <v>47</v>
+      </c>
+      <c r="W287" t="s">
+        <v>1774</v>
+      </c>
       <c r="X287" t="s">
         <v>71</v>
       </c>
@@ -32185,11 +32240,11 @@
       <c r="AA287" t="s">
         <v>52</v>
       </c>
-      <c r="AB287" t="s">
-        <v>50</v>
-      </c>
-      <c r="AC287" t="s">
-        <v>53</v>
+      <c r="AB287">
+        <v>3</v>
+      </c>
+      <c r="AC287">
+        <v>3</v>
       </c>
       <c r="AD287" t="s">
         <v>53</v>
@@ -32198,6 +32253,347 @@
         <v>3</v>
       </c>
       <c r="AF287" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="288" spans="1:32">
+      <c r="A288" t="s">
+        <v>1738</v>
+      </c>
+      <c r="B288" t="s">
+        <v>1739</v>
+      </c>
+      <c r="C288" t="s">
+        <v>34</v>
+      </c>
+      <c r="D288" t="s">
+        <v>35</v>
+      </c>
+      <c r="E288" t="s">
+        <v>36</v>
+      </c>
+      <c r="F288" t="s">
+        <v>1775</v>
+      </c>
+      <c r="G288" t="s">
+        <v>1776</v>
+      </c>
+      <c r="J288" t="s">
+        <v>39</v>
+      </c>
+      <c r="K288" t="s">
+        <v>239</v>
+      </c>
+      <c r="L288" t="s">
+        <v>240</v>
+      </c>
+      <c r="M288" t="s">
+        <v>42</v>
+      </c>
+      <c r="N288" t="s">
+        <v>1777</v>
+      </c>
+      <c r="O288" t="s">
+        <v>1778</v>
+      </c>
+      <c r="P288" t="s">
+        <v>1779</v>
+      </c>
+      <c r="Q288">
+        <v>8</v>
+      </c>
+      <c r="R288">
+        <v>4.6</v>
+      </c>
+      <c r="S288" t="s">
+        <v>44</v>
+      </c>
+      <c r="T288" t="s">
+        <v>1780</v>
+      </c>
+      <c r="U288" t="s">
+        <v>1781</v>
+      </c>
+      <c r="V288" t="s">
+        <v>47</v>
+      </c>
+      <c r="W288" t="s">
+        <v>1782</v>
+      </c>
+      <c r="X288" t="s">
+        <v>49</v>
+      </c>
+      <c r="Y288">
+        <v>4</v>
+      </c>
+      <c r="Z288">
+        <v>2</v>
+      </c>
+      <c r="AA288" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB288">
+        <v>3</v>
+      </c>
+      <c r="AC288" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD288" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE288">
+        <v>4</v>
+      </c>
+      <c r="AF288" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="289" spans="1:32">
+      <c r="A289" t="s">
+        <v>1738</v>
+      </c>
+      <c r="B289" t="s">
+        <v>1739</v>
+      </c>
+      <c r="C289" t="s">
+        <v>34</v>
+      </c>
+      <c r="D289" t="s">
+        <v>35</v>
+      </c>
+      <c r="E289" t="s">
+        <v>36</v>
+      </c>
+      <c r="F289" t="s">
+        <v>1783</v>
+      </c>
+      <c r="G289" t="s">
+        <v>1784</v>
+      </c>
+      <c r="J289" t="s">
+        <v>53</v>
+      </c>
+      <c r="K289" t="s">
+        <v>351</v>
+      </c>
+      <c r="L289" t="s">
+        <v>352</v>
+      </c>
+      <c r="M289" t="s">
+        <v>42</v>
+      </c>
+      <c r="N289" t="s">
+        <v>1785</v>
+      </c>
+      <c r="O289" t="s">
+        <v>1786</v>
+      </c>
+      <c r="P289" t="s">
+        <v>1787</v>
+      </c>
+      <c r="Q289">
+        <v>22</v>
+      </c>
+      <c r="R289">
+        <v>4.7</v>
+      </c>
+      <c r="S289" t="s">
+        <v>44</v>
+      </c>
+      <c r="T289" t="s">
+        <v>985</v>
+      </c>
+      <c r="U289" t="s">
+        <v>1788</v>
+      </c>
+      <c r="V289" t="s">
+        <v>47</v>
+      </c>
+      <c r="W289" t="s">
+        <v>1789</v>
+      </c>
+      <c r="X289" t="s">
+        <v>49</v>
+      </c>
+      <c r="Y289">
+        <v>3</v>
+      </c>
+      <c r="Z289">
+        <v>2</v>
+      </c>
+      <c r="AA289">
+        <v>2</v>
+      </c>
+      <c r="AB289">
+        <v>4</v>
+      </c>
+      <c r="AC289" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD289" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE289">
+        <v>3</v>
+      </c>
+      <c r="AF289" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="290" spans="1:32">
+      <c r="A290" t="s">
+        <v>1738</v>
+      </c>
+      <c r="B290" t="s">
+        <v>1739</v>
+      </c>
+      <c r="C290" t="s">
+        <v>34</v>
+      </c>
+      <c r="D290" t="s">
+        <v>35</v>
+      </c>
+      <c r="E290" t="s">
+        <v>36</v>
+      </c>
+      <c r="F290" t="s">
+        <v>1790</v>
+      </c>
+      <c r="G290" t="s">
+        <v>1791</v>
+      </c>
+      <c r="J290" t="s">
+        <v>53</v>
+      </c>
+      <c r="K290" t="s">
+        <v>193</v>
+      </c>
+      <c r="L290" t="s">
+        <v>194</v>
+      </c>
+      <c r="M290" t="s">
+        <v>42</v>
+      </c>
+      <c r="N290" t="s">
+        <v>1792</v>
+      </c>
+      <c r="O290" t="s">
+        <v>1793</v>
+      </c>
+      <c r="P290" t="s">
+        <v>1794</v>
+      </c>
+      <c r="Q290">
+        <v>33</v>
+      </c>
+      <c r="R290">
+        <v>4.6</v>
+      </c>
+      <c r="S290" t="s">
+        <v>44</v>
+      </c>
+      <c r="T290" t="s">
+        <v>1795</v>
+      </c>
+      <c r="U290" t="s">
+        <v>1796</v>
+      </c>
+      <c r="V290" t="s">
+        <v>47</v>
+      </c>
+      <c r="W290" t="s">
+        <v>1797</v>
+      </c>
+      <c r="X290" t="s">
+        <v>49</v>
+      </c>
+      <c r="Y290">
+        <v>3</v>
+      </c>
+      <c r="Z290" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA290" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB290" t="s">
+        <v>50</v>
+      </c>
+      <c r="AC290" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD290" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE290">
+        <v>3</v>
+      </c>
+      <c r="AF290" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="291" spans="1:32">
+      <c r="A291" t="s">
+        <v>1738</v>
+      </c>
+      <c r="B291" t="s">
+        <v>1739</v>
+      </c>
+      <c r="C291" t="s">
+        <v>34</v>
+      </c>
+      <c r="D291" t="s">
+        <v>35</v>
+      </c>
+      <c r="E291" t="s">
+        <v>36</v>
+      </c>
+      <c r="F291" t="s">
+        <v>1798</v>
+      </c>
+      <c r="G291" t="s">
+        <v>1799</v>
+      </c>
+      <c r="J291" t="s">
+        <v>53</v>
+      </c>
+      <c r="K291" t="s">
+        <v>66</v>
+      </c>
+      <c r="L291" t="s">
+        <v>67</v>
+      </c>
+      <c r="M291" t="s">
+        <v>42</v>
+      </c>
+      <c r="N291" t="s">
+        <v>436</v>
+      </c>
+      <c r="X291" t="s">
+        <v>71</v>
+      </c>
+      <c r="Y291">
+        <v>3</v>
+      </c>
+      <c r="Z291" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA291" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB291" t="s">
+        <v>50</v>
+      </c>
+      <c r="AC291" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD291" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE291">
+        <v>3</v>
+      </c>
+      <c r="AF291" t="s">
         <v>437</v>
       </c>
     </row>
@@ -32208,5 +32604,8 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:AF263 A264:T264 V264:AF265 A265:P265 S265 A266:AF291" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>